<commit_message>
Excel: restyle Outcome Type and P/DO tabs to match other sheets
Also dedupe Outcome Type to 60 abstracts; highlight P/DO note rows.
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -120,8 +120,18 @@
     <font>
       <i val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -181,8 +191,23 @@
         <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B2A4A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F7F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -220,11 +245,25 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -296,6 +335,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -661,1746 +713,1479 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="B2:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="38" t="inlineStr">
+    <row r="2">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>Outcome Type Coding — PSAU Corpus (60 abstracts)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Coded from abstract results language. Categories: Binary (presence/absence, diagnostic pos/neg, yes/no); Continuous (means, yields, rates); Mixed; Null/NS (explicit non-significance); Other.</t>
-        </is>
-      </c>
-    </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Draft_004 — outcome type coding for the 60-abstract PSAU corpus.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="39" t="inlineStr">
+      <c r="B3" s="43" t="inlineStr">
+        <is>
+          <t>Coded from abstract results language. Categories: Binary · Continuous · Mixed · Null/NS · Other. One row per abstract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="44" t="inlineStr">
         <is>
           <t>Abstract ID</t>
         </is>
       </c>
-      <c r="B4" s="39" t="inlineStr">
+      <c r="C5" s="44" t="inlineStr">
         <is>
           <t>Discipline</t>
         </is>
       </c>
-      <c r="C4" s="39" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>Hedges</t>
         </is>
       </c>
-      <c r="D4" s="39" t="inlineStr">
+      <c r="E5" s="44" t="inlineStr">
         <is>
           <t>Outcome Type</t>
         </is>
       </c>
-      <c r="E4" s="39" t="inlineStr">
+      <c r="F5" s="44" t="inlineStr">
         <is>
           <t>Coder Notes</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="40" t="inlineStr">
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="45" t="inlineStr">
+        <is>
+          <t>Acs1</t>
+        </is>
+      </c>
+      <c r="C6" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D6" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="45" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="F6" s="45" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>Acs10</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D7" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F7" s="46" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="45" t="inlineStr">
+        <is>
+          <t>Acs2</t>
+        </is>
+      </c>
+      <c r="C8" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D8" s="45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="45" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="inlineStr">
+        <is>
+          <t>NS language; rescue-hedging pattern (sig not observed but potential benefits)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>Acs3</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D9" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F9" s="46" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="45" t="inlineStr">
+        <is>
+          <t>Acs4</t>
+        </is>
+      </c>
+      <c r="C10" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="45" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>Acs5</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D11" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="46" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="F11" s="46" t="inlineStr">
+        <is>
+          <t>sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="45" t="inlineStr">
+        <is>
+          <t>Acs6</t>
+        </is>
+      </c>
+      <c r="C12" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D12" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="F12" s="45" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="46" t="inlineStr">
+        <is>
+          <t>Acs7</t>
+        </is>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D13" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F13" s="46" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="45" t="inlineStr">
+        <is>
+          <t>Acs8</t>
+        </is>
+      </c>
+      <c r="C14" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D14" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="45" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F14" s="45" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>Acs9</t>
+        </is>
+      </c>
+      <c r="C15" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D15" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F15" s="46" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="45" t="inlineStr">
+        <is>
+          <t>Aas1</t>
+        </is>
+      </c>
+      <c r="C16" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D16" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="45" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F16" s="45" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>Aas10</t>
+        </is>
+      </c>
+      <c r="C17" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D17" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F17" s="46" t="inlineStr">
+        <is>
+          <t>NS language; sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="45" t="inlineStr">
+        <is>
+          <t>Aas2</t>
+        </is>
+      </c>
+      <c r="C18" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D18" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="45" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="F18" s="45" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="46" t="inlineStr">
+        <is>
+          <t>Aas3</t>
+        </is>
+      </c>
+      <c r="C19" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D19" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F19" s="46" t="inlineStr">
+        <is>
+          <t>NS language; sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="45" t="inlineStr">
+        <is>
+          <t>Aas4</t>
+        </is>
+      </c>
+      <c r="C20" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D20" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="45" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F20" s="45" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="46" t="inlineStr">
+        <is>
+          <t>Aas5</t>
+        </is>
+      </c>
+      <c r="C21" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D21" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="46" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="F21" s="46" t="inlineStr">
+        <is>
+          <t>sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="45" t="inlineStr">
+        <is>
+          <t>Aas6</t>
+        </is>
+      </c>
+      <c r="C22" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D22" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="45" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F22" s="45" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t>Aas7</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D23" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F23" s="46" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="45" t="inlineStr">
+        <is>
+          <t>Aas8</t>
+        </is>
+      </c>
+      <c r="C24" s="45" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D24" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="F24" s="45" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t>Aas9</t>
+        </is>
+      </c>
+      <c r="C25" s="46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D25" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F25" s="46" t="inlineStr">
+        <is>
+          <t>NS language; sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="45" t="inlineStr">
+        <is>
+          <t>VM1</t>
+        </is>
+      </c>
+      <c r="C26" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D26" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="45" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F26" s="45" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="B27" s="46" t="inlineStr">
+        <is>
+          <t>VM2</t>
+        </is>
+      </c>
+      <c r="C27" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D27" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="46" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F27" s="46" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="45" t="inlineStr">
+        <is>
+          <t>VM3</t>
+        </is>
+      </c>
+      <c r="C28" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D28" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="45" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="F28" s="45" t="inlineStr">
+        <is>
+          <t>diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="46" t="inlineStr">
+        <is>
+          <t>VM4</t>
+        </is>
+      </c>
+      <c r="C29" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D29" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="46" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="F29" s="46" t="inlineStr">
+        <is>
+          <t>diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="45" t="inlineStr">
+        <is>
+          <t>VM5</t>
+        </is>
+      </c>
+      <c r="C30" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D30" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="F30" s="45" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="46" t="inlineStr">
+        <is>
+          <t>VM6</t>
+        </is>
+      </c>
+      <c r="C31" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D31" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F31" s="46" t="inlineStr">
+        <is>
+          <t>NS language; sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="45" t="inlineStr">
+        <is>
+          <t>VM7</t>
+        </is>
+      </c>
+      <c r="C32" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D32" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="45" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="F32" s="45" t="inlineStr">
+        <is>
+          <t>diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="B33" s="46" t="inlineStr">
+        <is>
+          <t>VM8</t>
+        </is>
+      </c>
+      <c r="C33" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D33" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="46" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="F33" s="46" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="B34" s="45" t="inlineStr">
+        <is>
+          <t>VM9</t>
+        </is>
+      </c>
+      <c r="C34" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D34" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="45" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="F34" s="45" t="inlineStr">
+        <is>
+          <t>diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="B35" s="46" t="inlineStr">
+        <is>
+          <t>VM10</t>
+        </is>
+      </c>
+      <c r="C35" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D35" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="46" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="F35" s="46" t="inlineStr">
+        <is>
+          <t>diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="B36" s="45" t="inlineStr">
+        <is>
+          <t>VM11</t>
+        </is>
+      </c>
+      <c r="C36" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D36" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="45" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="F36" s="45" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="46" t="inlineStr">
+        <is>
+          <t>VM12</t>
+        </is>
+      </c>
+      <c r="C37" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D37" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="46" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="F37" s="46" t="inlineStr">
+        <is>
+          <t>diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="B38" s="45" t="inlineStr">
+        <is>
+          <t>VM13</t>
+        </is>
+      </c>
+      <c r="C38" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D38" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="45" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="F38" s="45" t="inlineStr">
+        <is>
+          <t>sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t>VM14</t>
+        </is>
+      </c>
+      <c r="C39" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D39" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="46" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="B40" s="45" t="inlineStr">
+        <is>
+          <t>VM15</t>
+        </is>
+      </c>
+      <c r="C40" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D40" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="F40" s="45" t="n"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t>VM16</t>
+        </is>
+      </c>
+      <c r="C41" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D41" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="46" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F41" s="46" t="inlineStr">
+        <is>
+          <t>NS language; sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="B42" s="45" t="inlineStr">
+        <is>
+          <t>VM17</t>
+        </is>
+      </c>
+      <c r="C42" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D42" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="45" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="F42" s="45" t="inlineStr">
+        <is>
+          <t>sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="B43" s="46" t="inlineStr">
+        <is>
+          <t>VM18</t>
+        </is>
+      </c>
+      <c r="C43" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D43" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="46" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="F43" s="46" t="inlineStr">
+        <is>
+          <t>sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="B44" s="45" t="inlineStr">
+        <is>
+          <t>VM19</t>
+        </is>
+      </c>
+      <c r="C44" s="45" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D44" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="45" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="F44" s="45" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="B45" s="46" t="inlineStr">
+        <is>
+          <t>VM20</t>
+        </is>
+      </c>
+      <c r="C45" s="46" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="D45" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="46" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="F45" s="46" t="inlineStr">
+        <is>
+          <t>sig language</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="B46" s="45" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="B5" s="40" t="inlineStr">
+      <c r="C46" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C5" s="40" t="n">
+      <c r="D46" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="40" t="inlineStr">
+      <c r="E46" s="45" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="E5" s="40" t="inlineStr">
+      <c r="F46" s="45" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="40" t="inlineStr">
+    <row r="47" ht="22" customHeight="1">
+      <c r="B47" s="46" t="inlineStr">
         <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="B6" s="40" t="inlineStr">
+      <c r="C47" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C6" s="40" t="n">
+      <c r="D47" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="40" t="inlineStr">
+      <c r="E47" s="46" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="E6" s="40" t="inlineStr">
+      <c r="F47" s="46" t="inlineStr">
         <is>
           <t>no zone of inhibition / did not possess</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="40" t="inlineStr">
+    <row r="48" ht="22" customHeight="1">
+      <c r="B48" s="45" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
-      <c r="B7" s="40" t="inlineStr">
+      <c r="C48" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C7" s="40" t="n">
+      <c r="D48" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="40" t="inlineStr">
+      <c r="E48" s="45" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="E7" s="40" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="40" t="inlineStr">
+      <c r="F48" s="45" t="n"/>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="B49" s="46" t="inlineStr">
         <is>
           <t>B4</t>
         </is>
       </c>
-      <c r="B8" s="40" t="inlineStr">
+      <c r="C49" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C8" s="40" t="n">
+      <c r="D49" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="40" t="inlineStr">
+      <c r="E49" s="46" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E8" s="40" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="F49" s="46" t="n"/>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="B50" s="45" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="C50" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C9" s="40" t="n">
+      <c r="D50" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="E50" s="45" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="E9" s="40" t="inlineStr">
+      <c r="F50" s="45" t="inlineStr">
         <is>
           <t>NS language; sig language</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="40" t="inlineStr">
+    <row r="51" ht="22" customHeight="1">
+      <c r="B51" s="46" t="inlineStr">
         <is>
           <t>B6</t>
         </is>
       </c>
-      <c r="B10" s="40" t="inlineStr">
+      <c r="C51" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C10" s="40" t="n">
+      <c r="D51" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="40" t="inlineStr">
+      <c r="E51" s="46" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="E10" s="40" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="40" t="inlineStr">
+      <c r="F51" s="46" t="n"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="B52" s="45" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="B11" s="40" t="inlineStr">
+      <c r="C52" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C11" s="40" t="n">
+      <c r="D52" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="40" t="inlineStr">
+      <c r="E52" s="45" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E11" s="40" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="40" t="inlineStr">
+      <c r="F52" s="45" t="n"/>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="B53" s="46" t="inlineStr">
         <is>
           <t>B8</t>
         </is>
       </c>
-      <c r="B12" s="40" t="inlineStr">
+      <c r="C53" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C12" s="40" t="n">
+      <c r="D53" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="40" t="inlineStr">
+      <c r="E53" s="46" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="E12" s="40" t="inlineStr">
+      <c r="F53" s="46" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="40" t="inlineStr">
+    <row r="54" ht="22" customHeight="1">
+      <c r="B54" s="45" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="B13" s="40" t="inlineStr">
+      <c r="C54" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C13" s="40" t="n">
+      <c r="D54" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="40" t="inlineStr">
+      <c r="E54" s="45" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="E13" s="40" t="inlineStr">
+      <c r="F54" s="45" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="40" t="inlineStr">
+    <row r="55" ht="22" customHeight="1">
+      <c r="B55" s="46" t="inlineStr">
         <is>
           <t>B10</t>
         </is>
       </c>
-      <c r="B14" s="40" t="inlineStr">
+      <c r="C55" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C14" s="40" t="n">
+      <c r="D55" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="40" t="inlineStr">
+      <c r="E55" s="46" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E14" s="40" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="40" t="inlineStr">
+      <c r="F55" s="46" t="n"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="B56" s="45" t="inlineStr">
         <is>
           <t>B11</t>
         </is>
       </c>
-      <c r="B15" s="40" t="inlineStr">
+      <c r="C56" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C15" s="40" t="n">
+      <c r="D56" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="40" t="inlineStr">
+      <c r="E56" s="45" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="E15" s="40" t="inlineStr">
+      <c r="F56" s="45" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="40" t="inlineStr">
+    <row r="57" ht="22" customHeight="1">
+      <c r="B57" s="46" t="inlineStr">
         <is>
           <t>B12</t>
         </is>
       </c>
-      <c r="B16" s="40" t="inlineStr">
+      <c r="C57" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C16" s="40" t="n">
+      <c r="D57" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="40" t="inlineStr">
+      <c r="E57" s="46" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="E16" s="40" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="40" t="inlineStr">
+      <c r="F57" s="46" t="n"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="B58" s="45" t="inlineStr">
         <is>
           <t>B13</t>
         </is>
       </c>
-      <c r="B17" s="40" t="inlineStr">
+      <c r="C58" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C17" s="40" t="n">
+      <c r="D58" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="40" t="inlineStr">
+      <c r="E58" s="45" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="E17" s="40" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="40" t="inlineStr">
+      <c r="F58" s="45" t="n"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="B59" s="46" t="inlineStr">
         <is>
           <t>B14</t>
         </is>
       </c>
-      <c r="B18" s="40" t="inlineStr">
+      <c r="C59" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C18" s="40" t="n">
+      <c r="D59" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="D18" s="40" t="inlineStr">
+      <c r="E59" s="46" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E18" s="40" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="40" t="inlineStr">
+      <c r="F59" s="46" t="n"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="B60" s="45" t="inlineStr">
         <is>
           <t>B15</t>
         </is>
       </c>
-      <c r="B19" s="40" t="inlineStr">
+      <c r="C60" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C19" s="40" t="n">
+      <c r="D60" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="40" t="inlineStr">
+      <c r="E60" s="45" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="E19" s="40" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="40" t="inlineStr">
+      <c r="F60" s="45" t="n"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="B61" s="46" t="inlineStr">
         <is>
           <t>B16</t>
         </is>
       </c>
-      <c r="B20" s="40" t="inlineStr">
+      <c r="C61" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C20" s="40" t="n">
+      <c r="D61" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="D20" s="40" t="inlineStr">
+      <c r="E61" s="46" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="E20" s="40" t="inlineStr">
+      <c r="F61" s="46" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="40" t="inlineStr">
+    <row r="62" ht="22" customHeight="1">
+      <c r="B62" s="45" t="inlineStr">
         <is>
           <t>B17</t>
         </is>
       </c>
-      <c r="B21" s="40" t="inlineStr">
+      <c r="C62" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C21" s="40" t="n">
+      <c r="D62" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="D21" s="40" t="inlineStr">
+      <c r="E62" s="45" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="E21" s="40" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="F62" s="45" t="n"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="B63" s="46" t="inlineStr">
         <is>
           <t>B18</t>
         </is>
       </c>
-      <c r="B22" s="40" t="inlineStr">
+      <c r="C63" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C22" s="40" t="n">
+      <c r="D63" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="40" t="inlineStr">
+      <c r="E63" s="46" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="E22" s="40" t="inlineStr">
+      <c r="F63" s="46" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="40" t="inlineStr">
+    <row r="64" ht="22" customHeight="1">
+      <c r="B64" s="45" t="inlineStr">
         <is>
           <t>B19</t>
         </is>
       </c>
-      <c r="B23" s="40" t="inlineStr">
+      <c r="C64" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C23" s="40" t="n">
+      <c r="D64" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="40" t="inlineStr">
+      <c r="E64" s="45" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="E23" s="40" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="40" t="inlineStr">
+      <c r="F64" s="45" t="n"/>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="B65" s="46" t="inlineStr">
         <is>
           <t>B20</t>
         </is>
       </c>
-      <c r="B24" s="40" t="inlineStr">
+      <c r="C65" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C24" s="40" t="n">
+      <c r="D65" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="40" t="inlineStr">
+      <c r="E65" s="46" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="E24" s="40" t="inlineStr">
+      <c r="F65" s="46" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="40" t="inlineStr">
-        <is>
-          <t>VM1</t>
-        </is>
-      </c>
-      <c r="B25" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C25" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="40" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="E25" s="40" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="40" t="inlineStr">
-        <is>
-          <t>VM2</t>
-        </is>
-      </c>
-      <c r="B26" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C26" s="40" t="n">
-        <v>3</v>
-      </c>
-      <c r="D26" s="40" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="E26" s="40" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="40" t="inlineStr">
-        <is>
-          <t>VM3</t>
-        </is>
-      </c>
-      <c r="B27" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C27" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="40" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="E27" s="40" t="inlineStr">
-        <is>
-          <t>diagnostic</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="40" t="inlineStr">
-        <is>
-          <t>VM4</t>
-        </is>
-      </c>
-      <c r="B28" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C28" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="40" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="E28" s="40" t="inlineStr">
-        <is>
-          <t>diagnostic</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="40" t="inlineStr">
-        <is>
-          <t>VM5</t>
-        </is>
-      </c>
-      <c r="B29" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C29" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="40" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="E29" s="40" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="40" t="inlineStr">
-        <is>
-          <t>VM6</t>
-        </is>
-      </c>
-      <c r="B30" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C30" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E30" s="40" t="inlineStr">
-        <is>
-          <t>NS language; sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="40" t="inlineStr">
-        <is>
-          <t>VM7</t>
-        </is>
-      </c>
-      <c r="B31" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C31" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="40" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="E31" s="40" t="inlineStr">
-        <is>
-          <t>diagnostic</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="40" t="inlineStr">
-        <is>
-          <t>VM8</t>
-        </is>
-      </c>
-      <c r="B32" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C32" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="40" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="E32" s="40" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="40" t="inlineStr">
-        <is>
-          <t>VM9</t>
-        </is>
-      </c>
-      <c r="B33" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C33" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="40" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="E33" s="40" t="inlineStr">
-        <is>
-          <t>diagnostic</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="40" t="inlineStr">
-        <is>
-          <t>VM10</t>
-        </is>
-      </c>
-      <c r="B34" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C34" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="40" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="E34" s="40" t="inlineStr">
-        <is>
-          <t>diagnostic</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="40" t="inlineStr">
-        <is>
-          <t>VM11</t>
-        </is>
-      </c>
-      <c r="B35" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C35" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="40" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="E35" s="40" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="40" t="inlineStr">
-        <is>
-          <t>VM12</t>
-        </is>
-      </c>
-      <c r="B36" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C36" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="40" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="E36" s="40" t="inlineStr">
-        <is>
-          <t>diagnostic</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="40" t="inlineStr">
-        <is>
-          <t>VM13</t>
-        </is>
-      </c>
-      <c r="B37" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C37" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="40" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="E37" s="40" t="inlineStr">
-        <is>
-          <t>sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="40" t="inlineStr">
-        <is>
-          <t>VM14</t>
-        </is>
-      </c>
-      <c r="B38" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C38" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="40" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="E38" s="40" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="40" t="inlineStr">
-        <is>
-          <t>VM15</t>
-        </is>
-      </c>
-      <c r="B39" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C39" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="40" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="E39" s="40" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="40" t="inlineStr">
-        <is>
-          <t>VM16</t>
-        </is>
-      </c>
-      <c r="B40" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C40" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E40" s="40" t="inlineStr">
-        <is>
-          <t>NS language; sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="40" t="inlineStr">
-        <is>
-          <t>VM17</t>
-        </is>
-      </c>
-      <c r="B41" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C41" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="40" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="E41" s="40" t="inlineStr">
-        <is>
-          <t>sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="40" t="inlineStr">
-        <is>
-          <t>VM18</t>
-        </is>
-      </c>
-      <c r="B42" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C42" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" s="40" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="E42" s="40" t="inlineStr">
-        <is>
-          <t>sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="40" t="inlineStr">
-        <is>
-          <t>VM19</t>
-        </is>
-      </c>
-      <c r="B43" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C43" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" s="40" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="E43" s="40" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="40" t="inlineStr">
-        <is>
-          <t>VM20</t>
-        </is>
-      </c>
-      <c r="B44" s="40" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C44" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" s="40" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="E44" s="40" t="inlineStr">
-        <is>
-          <t>sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="40" t="inlineStr">
-        <is>
-          <t>Acs1</t>
-        </is>
-      </c>
-      <c r="B45" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C45" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="40" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="E45" s="40" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="40" t="inlineStr">
-        <is>
-          <t>Acs2</t>
-        </is>
-      </c>
-      <c r="B46" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C46" s="40" t="n">
-        <v>8</v>
-      </c>
-      <c r="D46" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E46" s="40" t="inlineStr">
-        <is>
-          <t>NS language; rescue-hedging pattern (sig not observed but potential benefits)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="40" t="inlineStr">
-        <is>
-          <t>Acs3</t>
-        </is>
-      </c>
-      <c r="B47" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C47" s="40" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E47" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="40" t="inlineStr">
-        <is>
-          <t>Acs4</t>
-        </is>
-      </c>
-      <c r="B48" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C48" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E48" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="40" t="inlineStr">
-        <is>
-          <t>Acs5</t>
-        </is>
-      </c>
-      <c r="B49" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C49" s="40" t="n">
-        <v>2</v>
-      </c>
-      <c r="D49" s="40" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="E49" s="40" t="inlineStr">
-        <is>
-          <t>sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="40" t="inlineStr">
-        <is>
-          <t>Acs6</t>
-        </is>
-      </c>
-      <c r="B50" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C50" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="40" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="E50" s="40" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="40" t="inlineStr">
-        <is>
-          <t>Acs7</t>
-        </is>
-      </c>
-      <c r="B51" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C51" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E51" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="40" t="inlineStr">
-        <is>
-          <t>Acs8</t>
-        </is>
-      </c>
-      <c r="B52" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C52" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E52" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="40" t="inlineStr">
-        <is>
-          <t>Acs9</t>
-        </is>
-      </c>
-      <c r="B53" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C53" s="40" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E53" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="40" t="inlineStr">
-        <is>
-          <t>Acs10</t>
-        </is>
-      </c>
-      <c r="B54" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C54" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E54" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="40" t="inlineStr">
-        <is>
-          <t>Aas1</t>
-        </is>
-      </c>
-      <c r="B55" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C55" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E55" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="40" t="inlineStr">
-        <is>
-          <t>Aas2</t>
-        </is>
-      </c>
-      <c r="B56" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C56" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="40" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="E56" s="40" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="40" t="inlineStr">
-        <is>
-          <t>Aas3</t>
-        </is>
-      </c>
-      <c r="B57" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C57" s="40" t="n">
-        <v>2</v>
-      </c>
-      <c r="D57" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E57" s="40" t="inlineStr">
-        <is>
-          <t>NS language; sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="40" t="inlineStr">
-        <is>
-          <t>Aas4</t>
-        </is>
-      </c>
-      <c r="B58" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C58" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E58" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="40" t="inlineStr">
-        <is>
-          <t>Aas5</t>
-        </is>
-      </c>
-      <c r="B59" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C59" s="40" t="n">
-        <v>2</v>
-      </c>
-      <c r="D59" s="40" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="E59" s="40" t="inlineStr">
-        <is>
-          <t>sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="40" t="inlineStr">
-        <is>
-          <t>Aas6</t>
-        </is>
-      </c>
-      <c r="B60" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C60" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D60" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E60" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="40" t="inlineStr">
-        <is>
-          <t>Aas7</t>
-        </is>
-      </c>
-      <c r="B61" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C61" s="40" t="n">
-        <v>3</v>
-      </c>
-      <c r="D61" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E61" s="40" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="40" t="inlineStr">
-        <is>
-          <t>Aas8</t>
-        </is>
-      </c>
-      <c r="B62" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C62" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D62" s="40" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="E62" s="40" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="40" t="inlineStr">
-        <is>
-          <t>Aas9</t>
-        </is>
-      </c>
-      <c r="B63" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C63" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E63" s="40" t="inlineStr">
-        <is>
-          <t>NS language; sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="40" t="inlineStr">
-        <is>
-          <t>Aas10</t>
-        </is>
-      </c>
-      <c r="B64" s="40" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C64" s="40" t="n">
-        <v>2</v>
-      </c>
-      <c r="D64" s="40" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="E64" s="40" t="inlineStr">
-        <is>
-          <t>NS language; sig language</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="37" t="inlineStr">
-        <is>
-          <t>Cross-tab: Outcome Type × Discipline (abstract counts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="41" t="inlineStr">
-        <is>
-          <t>Outcome Type</t>
-        </is>
-      </c>
-      <c r="B69" s="41" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C69" s="41" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="D69" s="41" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="E69" s="41" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="B70" t="n">
-        <v>0</v>
-      </c>
-      <c r="C70" t="n">
-        <v>8</v>
-      </c>
-      <c r="D70" t="n">
-        <v>7</v>
-      </c>
-      <c r="E70" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="B71" t="n">
-        <v>4</v>
-      </c>
-      <c r="C71" t="n">
-        <v>4</v>
-      </c>
-      <c r="D71" t="n">
-        <v>2</v>
-      </c>
-      <c r="E71" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="B72" t="n">
-        <v>2</v>
-      </c>
-      <c r="C72" t="n">
-        <v>3</v>
-      </c>
-      <c r="D72" t="n">
-        <v>4</v>
-      </c>
-      <c r="E72" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="B73" t="n">
-        <v>14</v>
-      </c>
-      <c r="C73" t="n">
-        <v>2</v>
-      </c>
-      <c r="D73" t="n">
-        <v>5</v>
-      </c>
-      <c r="E73" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B74" t="n">
-        <v>0</v>
-      </c>
-      <c r="C74" t="n">
-        <v>3</v>
-      </c>
-      <c r="D74" t="n">
-        <v>2</v>
-      </c>
-      <c r="E74" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B75" t="n">
-        <v>20</v>
-      </c>
-      <c r="C75" t="n">
-        <v>20</v>
-      </c>
-      <c r="D75" t="n">
-        <v>20</v>
-      </c>
-      <c r="E75" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="37" t="inlineStr">
-        <is>
-          <t>Mean hedges per abstract by Outcome Type × Discipline</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="41" t="inlineStr">
-        <is>
-          <t>Outcome Type</t>
-        </is>
-      </c>
-      <c r="B79" s="41" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C79" s="41" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="D79" s="41" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C80" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="D80" t="n">
-        <v>1.57</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="C81" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D81" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C82" t="n">
-        <v>1</v>
-      </c>
-      <c r="D82" t="n">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C83" t="n">
-        <v>0</v>
-      </c>
-      <c r="D83" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C84" t="n">
-        <v>1</v>
-      </c>
-      <c r="D84" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="42" t="inlineStr">
-        <is>
-          <t>Binary-outcome account of VM density is NOT supported: VM Binary mean 0.38 (n=8) vs Biology Binary mean 1.57 (n=7). VM low rate is a VM pattern, not a binary pattern. Clearer lead: Agriculture Null/NS 14/20 vs VM 2/20; Agri Null/NS mean ~1.5 hedges; Acs2 = null-rescue hedging.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Agri Null/NS n is high; Acs2 (Null/NS, 8 hedges) is the rescue-hedging outlier, not removed from outcome coding.</t>
-        </is>
-      </c>
+    <row r="66" ht="32" customHeight="1">
+      <c r="B66" s="46" t="n"/>
+      <c r="C66" s="46" t="n"/>
+      <c r="D66" s="46" t="n"/>
+      <c r="E66" s="46" t="n"/>
+      <c r="F66" s="46" t="n"/>
+    </row>
+    <row r="67" ht="32" customHeight="1">
+      <c r="B67" s="46" t="n"/>
+      <c r="C67" s="46" t="n"/>
+      <c r="D67" s="46" t="n"/>
+      <c r="E67" s="46" t="n"/>
+      <c r="F67" s="46" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2413,7 +2198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H101"/>
+  <dimension ref="B2:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2677,7 +2462,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -2777,8 +2561,6 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -11331,928 +11113,953 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="B2:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="37" t="inlineStr">
+    <row r="2">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>P and DO Functions — Scan Log (Non-Hedge Inventory)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="43" t="inlineStr">
+        <is>
+          <t>Discourse-organization connectors and politeness scan across 60 abstracts. Hedge? = N for all. Not counted in Layer 1/2 totals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="44" t="inlineStr">
         <is>
           <t>Abstract ID</t>
         </is>
       </c>
-      <c r="B1" s="37" t="inlineStr">
+      <c r="C5" s="44" t="inlineStr">
         <is>
           <t>Discipline</t>
         </is>
       </c>
-      <c r="C1" s="37" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>Phrase / Token</t>
         </is>
       </c>
-      <c r="D1" s="37" t="inlineStr">
+      <c r="E5" s="44" t="inlineStr">
         <is>
           <t>Context (short)</t>
         </is>
       </c>
-      <c r="E1" s="37" t="inlineStr">
-        <is>
-          <t>Function (EC/P/DO)</t>
-        </is>
-      </c>
-      <c r="F1" s="37" t="inlineStr">
-        <is>
-          <t>Hedge? (Y/N)</t>
-        </is>
-      </c>
-      <c r="G1" s="37" t="inlineStr">
+      <c r="F5" s="44" t="inlineStr">
+        <is>
+          <t>Function</t>
+        </is>
+      </c>
+      <c r="G5" s="44" t="inlineStr">
+        <is>
+          <t>Hedge?</t>
+        </is>
+      </c>
+      <c r="H5" s="44" t="inlineStr">
         <is>
           <t>Ambiguous</t>
         </is>
       </c>
-      <c r="H1" s="37" t="inlineStr">
+      <c r="I5" s="44" t="inlineStr">
         <is>
           <t>Reasoning</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="6" ht="32" customHeight="1">
+      <c r="B6" s="45" t="inlineStr">
         <is>
           <t>B6</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C6" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D6" s="45" t="inlineStr">
         <is>
           <t>Thus / Therefore</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E6" s="45" t="inlineStr">
         <is>
           <t>Thus, in the optimization process...; Therefore, further research will...</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F6" s="45" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G6" s="45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H6" s="45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I6" s="45" t="inlineStr">
         <is>
           <t>Move connectors (problem→method; limit→future work). Not epistemic hedges.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="46" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C7" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D7" s="46" t="inlineStr">
         <is>
           <t>Hence / thus</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E7" s="46" t="inlineStr">
         <is>
           <t>Hence, the biosynthesis is feasible; thus making a remarkable choice; thus demonstrating...</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F7" s="46" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G7" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H7" s="46" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I7" s="46" t="inlineStr">
         <is>
           <t>Claim-sequence connectors. Hedge if any is separate (may).</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="8" ht="32" customHeight="1">
+      <c r="B8" s="45" t="inlineStr">
         <is>
           <t>B10</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C8" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D8" s="45" t="inlineStr">
         <is>
           <t>Thus</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E8" s="45" t="inlineStr">
         <is>
           <t>Thus, the researcher provided a policy proposal...</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F8" s="45" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G8" s="45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H8" s="45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I8" s="45" t="inlineStr">
         <is>
           <t>Results→recommendation connector.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="9" ht="32" customHeight="1">
+      <c r="B9" s="46" t="inlineStr">
         <is>
           <t>B11</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C9" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D9" s="46" t="inlineStr">
         <is>
           <t>Hence</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E9" s="46" t="inlineStr">
         <is>
           <t>Hence, this study aimed to investigate...</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F9" s="46" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G9" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H9" s="46" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I9" s="46" t="inlineStr">
         <is>
           <t>Background→aim connector.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="10" ht="32" customHeight="1">
+      <c r="B10" s="45" t="inlineStr">
         <is>
           <t>B12</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D10" s="45" t="inlineStr">
         <is>
           <t>Hence</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E10" s="45" t="inlineStr">
         <is>
           <t>Hence, LAB have emerged as a focal point...</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F10" s="45" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G10" s="45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H10" s="45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I10" s="45" t="inlineStr">
         <is>
           <t>Problem→focus connector.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="11" ht="32" customHeight="1">
+      <c r="B11" s="46" t="inlineStr">
         <is>
           <t>B16</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C11" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D11" s="46" t="inlineStr">
         <is>
           <t>Thus / therefore</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E11" s="46" t="inlineStr">
         <is>
           <t>Thus, this study detected...; This study, therefore, underscores...</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F11" s="46" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G11" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H11" s="46" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I11" s="46" t="inlineStr">
         <is>
           <t>Rationale→aim / findings→implication connectors.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="12" ht="32" customHeight="1">
+      <c r="B12" s="45" t="inlineStr">
         <is>
           <t>B19</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D12" s="45" t="inlineStr">
         <is>
           <t>Hence / Thus</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E12" s="45" t="inlineStr">
         <is>
           <t>Hence, sustainable planning should...; Thus, local government should...</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F12" s="45" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G12" s="45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H12" s="45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I12" s="45" t="inlineStr">
         <is>
           <t>Problem/findings→recommendation connectors.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="13" ht="32" customHeight="1">
+      <c r="B13" s="46" t="inlineStr">
         <is>
           <t>B20</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C13" s="46" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D13" s="46" t="inlineStr">
         <is>
           <t>Therefore / Hence</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E13" s="46" t="inlineStr">
         <is>
           <t>Therefore, this study aims...; Hence, the study aimed...</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F13" s="46" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G13" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H13" s="46" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I13" s="46" t="inlineStr">
         <is>
           <t>Background→aim connectors.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="14" ht="32" customHeight="1">
+      <c r="B14" s="45" t="inlineStr">
         <is>
           <t>VM7</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C14" s="45" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D14" s="45" t="inlineStr">
         <is>
           <t>Thus</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E14" s="45" t="inlineStr">
         <is>
           <t>Thus, no significant association could be established</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F14" s="45" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G14" s="45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H14" s="45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I14" s="45" t="inlineStr">
         <is>
           <t>Results→conclusion connector.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="15" ht="32" customHeight="1">
+      <c r="B15" s="46" t="inlineStr">
         <is>
           <t>VM9</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C15" s="46" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D15" s="46" t="inlineStr">
         <is>
           <t>hence</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E15" s="46" t="inlineStr">
         <is>
           <t>hence, all individual shrimps counted as one sample</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F15" s="46" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G15" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H15" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I15" s="46" t="inlineStr">
         <is>
           <t>Methods sequencing only.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="16" ht="32" customHeight="1">
+      <c r="B16" s="45" t="inlineStr">
         <is>
           <t>VM12</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C16" s="45" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D16" s="45" t="inlineStr">
         <is>
           <t>Hence</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E16" s="45" t="inlineStr">
         <is>
           <t>Hence, this study aimed to detect ASF virus...</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F16" s="45" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G16" s="45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H16" s="45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I16" s="45" t="inlineStr">
         <is>
           <t>Background→aim connector.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="17" ht="32" customHeight="1">
+      <c r="B17" s="46" t="inlineStr">
         <is>
           <t>Acs5</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C17" s="46" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D17" s="46" t="inlineStr">
         <is>
           <t>Therefore</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E17" s="46" t="inlineStr">
         <is>
           <t>Therefore, the... (yield inference connector)</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F17" s="46" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G17" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H17" s="46" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I17" s="46" t="inlineStr">
         <is>
           <t>Results→inference connector.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="18" ht="32" customHeight="1">
+      <c r="B18" s="45" t="inlineStr">
         <is>
           <t>Aas9</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C18" s="45" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D18" s="45" t="inlineStr">
         <is>
           <t>Therefore</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E18" s="45" t="inlineStr">
         <is>
           <t>Therefore, it is recommended for future researchers...</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F18" s="45" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G18" s="45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H18" s="45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I18" s="45" t="inlineStr">
         <is>
           <t>Results→recommendation connector.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="19" ht="32" customHeight="1">
+      <c r="B19" s="46" t="inlineStr">
         <is>
           <t>Acs3</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C19" s="46" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D19" s="46" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E19" s="46" t="inlineStr">
         <is>
           <t>In conclusion, the number of rooted...</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F19" s="46" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G19" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H19" s="46" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I19" s="46" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="20" ht="32" customHeight="1">
+      <c r="B20" s="45" t="inlineStr">
         <is>
           <t>Acs7</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C20" s="45" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D20" s="45" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E20" s="45" t="inlineStr">
         <is>
           <t>In conclusion, the use of rice hull...</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F20" s="45" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G20" s="45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H20" s="45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I20" s="45" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="21" ht="32" customHeight="1">
+      <c r="B21" s="46" t="inlineStr">
         <is>
           <t>Acs10</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C21" s="46" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D21" s="46" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E21" s="46" t="inlineStr">
         <is>
           <t>In conclusion, T3:...</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F21" s="46" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G21" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H21" s="46" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I21" s="46" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="22" ht="32" customHeight="1">
+      <c r="B22" s="45" t="inlineStr">
         <is>
           <t>Aas3</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C22" s="45" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D22" s="45" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E22" s="45" t="inlineStr">
         <is>
           <t>In conclusion, proved the treatment 1...</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F22" s="45" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G22" s="45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H22" s="45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I22" s="45" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="23" ht="32" customHeight="1">
+      <c r="B23" s="46" t="inlineStr">
         <is>
           <t>Aas10</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C23" s="46" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D23" s="46" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E23" s="46" t="inlineStr">
         <is>
           <t>In conclusion, based on the results, it can be stated...</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F23" s="46" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G23" s="46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H23" s="46" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I23" s="46" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="24" ht="40" customHeight="1">
+      <c r="B24" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C24" s="47" t="inlineStr">
         <is>
           <t>All disciplines</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D24" s="47" t="inlineStr">
         <is>
           <t>(none)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E24" s="47" t="inlineStr">
         <is>
           <t>No "as X suggested", "in our view", "please", "kindly", "with due respect", "one might argue"</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F24" s="47" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G24" s="47" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H24" s="47" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I24" s="47" t="inlineStr">
         <is>
           <t>No politeness/deference devices in the 60 abstracts.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="25" ht="40" customHeight="1">
+      <c r="B25" s="47" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C25" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D25" s="47" t="inlineStr">
         <is>
           <t>regarding / with regard to / overall / first-second</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E25" s="47" t="inlineStr">
         <is>
           <t>Common in VM KAP and ranking sentences</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F25" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G25" s="47" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H25" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I25" s="47" t="inlineStr">
         <is>
           <t>Topic prepositions and ordinal ranking of results are NOT discourse-organization function. Left untagged.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="26" ht="40" customHeight="1">
+      <c r="B26" s="47" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C26" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D26" s="47" t="inlineStr">
         <is>
           <t>should / recommended (FP-Rec)</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E26" s="47" t="inlineStr">
         <is>
           <t>See Rejected Candidates</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F26" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G26" s="47" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H26" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I26" s="47" t="inlineStr">
         <is>
           <t>Deontic prescriptions. Reject reason FP-Rec, not Layer 2 P or DO.</t>
         </is>

</xml_diff>

<commit_message>
Excel: align remaining tab design (freeze, header row, subtitles, fonts)
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -130,6 +130,13 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font/>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="008C8A84"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="14">
     <fill>
@@ -207,7 +214,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -259,11 +266,12 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -346,6 +354,22 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2784,6 +2808,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="B3" s="48" t="inlineStr">
+        <is>
+          <t>Confirmed Layer 1 type + Layer 2 function codes for all retained hedges (n=65 tokens).</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -5654,6 +5685,13 @@
       <c r="B2" s="17" t="inlineStr">
         <is>
           <t>Rejected Hedge Candidates — False Positives</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="48" t="inlineStr">
+        <is>
+          <t>False-positive hedge candidates rejected under the Working Test, with reason codes.</t>
         </is>
       </c>
     </row>
@@ -7760,6 +7798,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="B3" s="48" t="inlineStr">
+        <is>
+          <t>Layer 3 optional unhedged assertion sites [R]/[G]/[C] (corpus-wide).</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -9103,7 +9148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F67"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9114,1468 +9159,1959 @@
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="49" t="n"/>
+      <c r="B1" s="49" t="n"/>
+      <c r="C1" s="49" t="n"/>
+      <c r="D1" s="49" t="n"/>
+      <c r="E1" s="49" t="n"/>
+      <c r="F1" s="49" t="n"/>
+      <c r="G1" s="49" t="n"/>
+      <c r="H1" s="49" t="n"/>
+      <c r="I1" s="49" t="n"/>
+      <c r="J1" s="49" t="n"/>
+      <c r="K1" s="49" t="n"/>
+      <c r="L1" s="49" t="n"/>
+    </row>
     <row r="2">
-      <c r="B2" s="17" t="inlineStr">
+      <c r="A2" s="49" t="n"/>
+      <c r="B2" s="50" t="inlineStr">
         <is>
           <t>Outcome Type Coding — PSAU Corpus (60 abstracts)</t>
         </is>
       </c>
+      <c r="C2" s="49" t="n"/>
+      <c r="D2" s="49" t="n"/>
+      <c r="E2" s="49" t="n"/>
+      <c r="F2" s="49" t="n"/>
+      <c r="G2" s="49" t="n"/>
+      <c r="H2" s="49" t="n"/>
+      <c r="I2" s="49" t="n"/>
+      <c r="J2" s="49" t="n"/>
+      <c r="K2" s="49" t="n"/>
+      <c r="L2" s="49" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="43" t="inlineStr">
+      <c r="A3" s="49" t="n"/>
+      <c r="B3" s="51" t="inlineStr">
         <is>
           <t>Coded from abstract results language. Categories: Binary · Continuous · Mixed · Null/NS · Other. One row per abstract.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="B5" s="44" t="inlineStr">
+      <c r="C3" s="49" t="n"/>
+      <c r="D3" s="49" t="n"/>
+      <c r="E3" s="49" t="n"/>
+      <c r="F3" s="49" t="n"/>
+      <c r="G3" s="49" t="n"/>
+      <c r="H3" s="49" t="n"/>
+      <c r="I3" s="49" t="n"/>
+      <c r="J3" s="49" t="n"/>
+      <c r="K3" s="49" t="n"/>
+      <c r="L3" s="49" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="49" t="n"/>
+      <c r="B4" s="52" t="inlineStr">
         <is>
           <t>Abstract ID</t>
         </is>
       </c>
-      <c r="C5" s="44" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>Discipline</t>
         </is>
       </c>
-      <c r="D5" s="44" t="inlineStr">
+      <c r="D4" s="52" t="inlineStr">
         <is>
           <t>Hedges</t>
         </is>
       </c>
-      <c r="E5" s="44" t="inlineStr">
+      <c r="E4" s="52" t="inlineStr">
         <is>
           <t>Outcome Type</t>
         </is>
       </c>
-      <c r="F5" s="44" t="inlineStr">
+      <c r="F4" s="52" t="inlineStr">
         <is>
           <t>Coder Notes</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="45" t="inlineStr">
+      <c r="G4" s="49" t="n"/>
+      <c r="H4" s="49" t="n"/>
+      <c r="I4" s="49" t="n"/>
+      <c r="J4" s="49" t="n"/>
+      <c r="K4" s="49" t="n"/>
+      <c r="L4" s="49" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="49" t="n"/>
+      <c r="B5" s="53" t="inlineStr">
         <is>
           <t>Acs1</t>
         </is>
       </c>
-      <c r="C6" s="45" t="inlineStr">
+      <c r="C5" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D6" s="45" t="n">
+      <c r="D5" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="45" t="inlineStr">
+      <c r="E5" s="53" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F6" s="45" t="n"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="46" t="inlineStr">
+      <c r="F5" s="53" t="n"/>
+      <c r="G5" s="49" t="n"/>
+      <c r="H5" s="49" t="n"/>
+      <c r="I5" s="49" t="n"/>
+      <c r="J5" s="49" t="n"/>
+      <c r="K5" s="49" t="n"/>
+      <c r="L5" s="49" t="n"/>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="49" t="n"/>
+      <c r="B6" s="54" t="inlineStr">
         <is>
           <t>Acs10</t>
         </is>
       </c>
-      <c r="C7" s="46" t="inlineStr">
+      <c r="C6" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D7" s="46" t="n">
+      <c r="D6" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="46" t="inlineStr">
+      <c r="E6" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F7" s="46" t="inlineStr">
+      <c r="F6" s="54" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="45" t="inlineStr">
+      <c r="G6" s="49" t="n"/>
+      <c r="H6" s="49" t="n"/>
+      <c r="I6" s="49" t="n"/>
+      <c r="J6" s="49" t="n"/>
+      <c r="K6" s="49" t="n"/>
+      <c r="L6" s="49" t="n"/>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="49" t="n"/>
+      <c r="B7" s="53" t="inlineStr">
         <is>
           <t>Acs2</t>
         </is>
       </c>
-      <c r="C8" s="45" t="inlineStr">
+      <c r="C7" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D8" s="45" t="n">
+      <c r="D7" s="53" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="45" t="inlineStr">
+      <c r="E7" s="53" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F8" s="45" t="inlineStr">
+      <c r="F7" s="53" t="inlineStr">
         <is>
           <t>NS language; rescue-hedging pattern (sig not observed but potential benefits)</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="46" t="inlineStr">
+      <c r="G7" s="49" t="n"/>
+      <c r="H7" s="49" t="n"/>
+      <c r="I7" s="49" t="n"/>
+      <c r="J7" s="49" t="n"/>
+      <c r="K7" s="49" t="n"/>
+      <c r="L7" s="49" t="n"/>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="49" t="n"/>
+      <c r="B8" s="54" t="inlineStr">
         <is>
           <t>Acs3</t>
         </is>
       </c>
-      <c r="C9" s="46" t="inlineStr">
+      <c r="C8" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D9" s="46" t="n">
+      <c r="D8" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="46" t="inlineStr">
+      <c r="E8" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F9" s="46" t="inlineStr">
+      <c r="F8" s="54" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="45" t="inlineStr">
+      <c r="G8" s="49" t="n"/>
+      <c r="H8" s="49" t="n"/>
+      <c r="I8" s="49" t="n"/>
+      <c r="J8" s="49" t="n"/>
+      <c r="K8" s="49" t="n"/>
+      <c r="L8" s="49" t="n"/>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="49" t="n"/>
+      <c r="B9" s="53" t="inlineStr">
         <is>
           <t>Acs4</t>
         </is>
       </c>
-      <c r="C10" s="45" t="inlineStr">
+      <c r="C9" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D10" s="45" t="n">
+      <c r="D9" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="45" t="inlineStr">
+      <c r="E9" s="53" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F10" s="45" t="inlineStr">
+      <c r="F9" s="53" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="46" t="inlineStr">
+      <c r="G9" s="49" t="n"/>
+      <c r="H9" s="49" t="n"/>
+      <c r="I9" s="49" t="n"/>
+      <c r="J9" s="49" t="n"/>
+      <c r="K9" s="49" t="n"/>
+      <c r="L9" s="49" t="n"/>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="49" t="n"/>
+      <c r="B10" s="54" t="inlineStr">
         <is>
           <t>Acs5</t>
         </is>
       </c>
-      <c r="C11" s="46" t="inlineStr">
+      <c r="C10" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D11" s="46" t="n">
+      <c r="D10" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="46" t="inlineStr">
+      <c r="E10" s="54" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F11" s="46" t="inlineStr">
+      <c r="F10" s="54" t="inlineStr">
         <is>
           <t>sig language</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="45" t="inlineStr">
+      <c r="G10" s="49" t="n"/>
+      <c r="H10" s="49" t="n"/>
+      <c r="I10" s="49" t="n"/>
+      <c r="J10" s="49" t="n"/>
+      <c r="K10" s="49" t="n"/>
+      <c r="L10" s="49" t="n"/>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="49" t="n"/>
+      <c r="B11" s="53" t="inlineStr">
         <is>
           <t>Acs6</t>
         </is>
       </c>
-      <c r="C12" s="45" t="inlineStr">
+      <c r="C11" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D12" s="45" t="n">
+      <c r="D11" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="45" t="inlineStr">
+      <c r="E11" s="53" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="F12" s="45" t="n"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="46" t="inlineStr">
+      <c r="F11" s="53" t="n"/>
+      <c r="G11" s="49" t="n"/>
+      <c r="H11" s="49" t="n"/>
+      <c r="I11" s="49" t="n"/>
+      <c r="J11" s="49" t="n"/>
+      <c r="K11" s="49" t="n"/>
+      <c r="L11" s="49" t="n"/>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="49" t="n"/>
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>Acs7</t>
         </is>
       </c>
-      <c r="C13" s="46" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D13" s="46" t="n">
+      <c r="D12" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="46" t="inlineStr">
+      <c r="E12" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F13" s="46" t="inlineStr">
+      <c r="F12" s="54" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="45" t="inlineStr">
+      <c r="G12" s="49" t="n"/>
+      <c r="H12" s="49" t="n"/>
+      <c r="I12" s="49" t="n"/>
+      <c r="J12" s="49" t="n"/>
+      <c r="K12" s="49" t="n"/>
+      <c r="L12" s="49" t="n"/>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="49" t="n"/>
+      <c r="B13" s="53" t="inlineStr">
         <is>
           <t>Acs8</t>
         </is>
       </c>
-      <c r="C14" s="45" t="inlineStr">
+      <c r="C13" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D14" s="45" t="n">
+      <c r="D13" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="45" t="inlineStr">
+      <c r="E13" s="53" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F14" s="45" t="inlineStr">
+      <c r="F13" s="53" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="46" t="inlineStr">
+      <c r="G13" s="49" t="n"/>
+      <c r="H13" s="49" t="n"/>
+      <c r="I13" s="49" t="n"/>
+      <c r="J13" s="49" t="n"/>
+      <c r="K13" s="49" t="n"/>
+      <c r="L13" s="49" t="n"/>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="49" t="n"/>
+      <c r="B14" s="54" t="inlineStr">
         <is>
           <t>Acs9</t>
         </is>
       </c>
-      <c r="C15" s="46" t="inlineStr">
+      <c r="C14" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D15" s="46" t="n">
+      <c r="D14" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="46" t="inlineStr">
+      <c r="E14" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F15" s="46" t="inlineStr">
+      <c r="F14" s="54" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="45" t="inlineStr">
+      <c r="G14" s="49" t="n"/>
+      <c r="H14" s="49" t="n"/>
+      <c r="I14" s="49" t="n"/>
+      <c r="J14" s="49" t="n"/>
+      <c r="K14" s="49" t="n"/>
+      <c r="L14" s="49" t="n"/>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="49" t="n"/>
+      <c r="B15" s="53" t="inlineStr">
         <is>
           <t>Aas1</t>
         </is>
       </c>
-      <c r="C16" s="45" t="inlineStr">
+      <c r="C15" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D16" s="45" t="n">
+      <c r="D15" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="45" t="inlineStr">
+      <c r="E15" s="53" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F16" s="45" t="inlineStr">
+      <c r="F15" s="53" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="46" t="inlineStr">
+      <c r="G15" s="49" t="n"/>
+      <c r="H15" s="49" t="n"/>
+      <c r="I15" s="49" t="n"/>
+      <c r="J15" s="49" t="n"/>
+      <c r="K15" s="49" t="n"/>
+      <c r="L15" s="49" t="n"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="49" t="n"/>
+      <c r="B16" s="54" t="inlineStr">
         <is>
           <t>Aas10</t>
         </is>
       </c>
-      <c r="C17" s="46" t="inlineStr">
+      <c r="C16" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D17" s="46" t="n">
+      <c r="D16" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="46" t="inlineStr">
+      <c r="E16" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F17" s="46" t="inlineStr">
+      <c r="F16" s="54" t="inlineStr">
         <is>
           <t>NS language; sig language</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="45" t="inlineStr">
+      <c r="G16" s="49" t="n"/>
+      <c r="H16" s="49" t="n"/>
+      <c r="I16" s="49" t="n"/>
+      <c r="J16" s="49" t="n"/>
+      <c r="K16" s="49" t="n"/>
+      <c r="L16" s="49" t="n"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="49" t="n"/>
+      <c r="B17" s="53" t="inlineStr">
         <is>
           <t>Aas2</t>
         </is>
       </c>
-      <c r="C18" s="45" t="inlineStr">
+      <c r="C17" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D18" s="45" t="n">
+      <c r="D17" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="45" t="inlineStr">
+      <c r="E17" s="53" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F18" s="45" t="n"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="46" t="inlineStr">
+      <c r="F17" s="53" t="n"/>
+      <c r="G17" s="49" t="n"/>
+      <c r="H17" s="49" t="n"/>
+      <c r="I17" s="49" t="n"/>
+      <c r="J17" s="49" t="n"/>
+      <c r="K17" s="49" t="n"/>
+      <c r="L17" s="49" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="49" t="n"/>
+      <c r="B18" s="54" t="inlineStr">
         <is>
           <t>Aas3</t>
         </is>
       </c>
-      <c r="C19" s="46" t="inlineStr">
+      <c r="C18" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D19" s="46" t="n">
+      <c r="D18" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="46" t="inlineStr">
+      <c r="E18" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F19" s="46" t="inlineStr">
+      <c r="F18" s="54" t="inlineStr">
         <is>
           <t>NS language; sig language</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="45" t="inlineStr">
+      <c r="G18" s="49" t="n"/>
+      <c r="H18" s="49" t="n"/>
+      <c r="I18" s="49" t="n"/>
+      <c r="J18" s="49" t="n"/>
+      <c r="K18" s="49" t="n"/>
+      <c r="L18" s="49" t="n"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="49" t="n"/>
+      <c r="B19" s="53" t="inlineStr">
         <is>
           <t>Aas4</t>
         </is>
       </c>
-      <c r="C20" s="45" t="inlineStr">
+      <c r="C19" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D20" s="45" t="n">
+      <c r="D19" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="45" t="inlineStr">
+      <c r="E19" s="53" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F20" s="45" t="inlineStr">
+      <c r="F19" s="53" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="46" t="inlineStr">
+      <c r="G19" s="49" t="n"/>
+      <c r="H19" s="49" t="n"/>
+      <c r="I19" s="49" t="n"/>
+      <c r="J19" s="49" t="n"/>
+      <c r="K19" s="49" t="n"/>
+      <c r="L19" s="49" t="n"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="49" t="n"/>
+      <c r="B20" s="54" t="inlineStr">
         <is>
           <t>Aas5</t>
         </is>
       </c>
-      <c r="C21" s="46" t="inlineStr">
+      <c r="C20" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D21" s="46" t="n">
+      <c r="D20" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E21" s="46" t="inlineStr">
+      <c r="E20" s="54" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F21" s="46" t="inlineStr">
+      <c r="F20" s="54" t="inlineStr">
         <is>
           <t>sig language</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="45" t="inlineStr">
+      <c r="G20" s="49" t="n"/>
+      <c r="H20" s="49" t="n"/>
+      <c r="I20" s="49" t="n"/>
+      <c r="J20" s="49" t="n"/>
+      <c r="K20" s="49" t="n"/>
+      <c r="L20" s="49" t="n"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="49" t="n"/>
+      <c r="B21" s="53" t="inlineStr">
         <is>
           <t>Aas6</t>
         </is>
       </c>
-      <c r="C22" s="45" t="inlineStr">
+      <c r="C21" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D22" s="45" t="n">
+      <c r="D21" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E22" s="45" t="inlineStr">
+      <c r="E21" s="53" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F22" s="45" t="inlineStr">
+      <c r="F21" s="53" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="46" t="inlineStr">
+      <c r="G21" s="49" t="n"/>
+      <c r="H21" s="49" t="n"/>
+      <c r="I21" s="49" t="n"/>
+      <c r="J21" s="49" t="n"/>
+      <c r="K21" s="49" t="n"/>
+      <c r="L21" s="49" t="n"/>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="49" t="n"/>
+      <c r="B22" s="54" t="inlineStr">
         <is>
           <t>Aas7</t>
         </is>
       </c>
-      <c r="C23" s="46" t="inlineStr">
+      <c r="C22" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D23" s="46" t="n">
+      <c r="D22" s="54" t="n">
         <v>3</v>
       </c>
-      <c r="E23" s="46" t="inlineStr">
+      <c r="E22" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F23" s="46" t="inlineStr">
+      <c r="F22" s="54" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="45" t="inlineStr">
+      <c r="G22" s="49" t="n"/>
+      <c r="H22" s="49" t="n"/>
+      <c r="I22" s="49" t="n"/>
+      <c r="J22" s="49" t="n"/>
+      <c r="K22" s="49" t="n"/>
+      <c r="L22" s="49" t="n"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="49" t="n"/>
+      <c r="B23" s="53" t="inlineStr">
         <is>
           <t>Aas8</t>
         </is>
       </c>
-      <c r="C24" s="45" t="inlineStr">
+      <c r="C23" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D24" s="45" t="n">
+      <c r="D23" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E24" s="45" t="inlineStr">
+      <c r="E23" s="53" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="F24" s="45" t="n"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="46" t="inlineStr">
+      <c r="F23" s="53" t="n"/>
+      <c r="G23" s="49" t="n"/>
+      <c r="H23" s="49" t="n"/>
+      <c r="I23" s="49" t="n"/>
+      <c r="J23" s="49" t="n"/>
+      <c r="K23" s="49" t="n"/>
+      <c r="L23" s="49" t="n"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="49" t="n"/>
+      <c r="B24" s="54" t="inlineStr">
         <is>
           <t>Aas9</t>
         </is>
       </c>
-      <c r="C25" s="46" t="inlineStr">
+      <c r="C24" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D25" s="46" t="n">
+      <c r="D24" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="46" t="inlineStr">
+      <c r="E24" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F25" s="46" t="inlineStr">
+      <c r="F24" s="54" t="inlineStr">
         <is>
           <t>NS language; sig language</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="45" t="inlineStr">
+      <c r="G24" s="49" t="n"/>
+      <c r="H24" s="49" t="n"/>
+      <c r="I24" s="49" t="n"/>
+      <c r="J24" s="49" t="n"/>
+      <c r="K24" s="49" t="n"/>
+      <c r="L24" s="49" t="n"/>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="49" t="n"/>
+      <c r="B25" s="53" t="inlineStr">
         <is>
           <t>VM1</t>
         </is>
       </c>
-      <c r="C26" s="45" t="inlineStr">
+      <c r="C25" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D26" s="45" t="n">
+      <c r="D25" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="45" t="inlineStr">
+      <c r="E25" s="53" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="F26" s="45" t="n"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="46" t="inlineStr">
+      <c r="F25" s="53" t="n"/>
+      <c r="G25" s="49" t="n"/>
+      <c r="H25" s="49" t="n"/>
+      <c r="I25" s="49" t="n"/>
+      <c r="J25" s="49" t="n"/>
+      <c r="K25" s="49" t="n"/>
+      <c r="L25" s="49" t="n"/>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="49" t="n"/>
+      <c r="B26" s="54" t="inlineStr">
         <is>
           <t>VM2</t>
         </is>
       </c>
-      <c r="C27" s="46" t="inlineStr">
+      <c r="C26" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D27" s="46" t="n">
+      <c r="D26" s="54" t="n">
         <v>3</v>
       </c>
-      <c r="E27" s="46" t="inlineStr">
+      <c r="E26" s="54" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="F27" s="46" t="n"/>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="45" t="inlineStr">
+      <c r="F26" s="54" t="n"/>
+      <c r="G26" s="49" t="n"/>
+      <c r="H26" s="49" t="n"/>
+      <c r="I26" s="49" t="n"/>
+      <c r="J26" s="49" t="n"/>
+      <c r="K26" s="49" t="n"/>
+      <c r="L26" s="49" t="n"/>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="49" t="n"/>
+      <c r="B27" s="53" t="inlineStr">
         <is>
           <t>VM3</t>
         </is>
       </c>
-      <c r="C28" s="45" t="inlineStr">
+      <c r="C27" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D28" s="45" t="n">
+      <c r="D27" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="45" t="inlineStr">
+      <c r="E27" s="53" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F28" s="45" t="inlineStr">
+      <c r="F27" s="53" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="46" t="inlineStr">
+      <c r="G27" s="49" t="n"/>
+      <c r="H27" s="49" t="n"/>
+      <c r="I27" s="49" t="n"/>
+      <c r="J27" s="49" t="n"/>
+      <c r="K27" s="49" t="n"/>
+      <c r="L27" s="49" t="n"/>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="49" t="n"/>
+      <c r="B28" s="54" t="inlineStr">
         <is>
           <t>VM4</t>
         </is>
       </c>
-      <c r="C29" s="46" t="inlineStr">
+      <c r="C28" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D29" s="46" t="n">
+      <c r="D28" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E29" s="46" t="inlineStr">
+      <c r="E28" s="54" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F29" s="46" t="inlineStr">
+      <c r="F28" s="54" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="45" t="inlineStr">
+      <c r="G28" s="49" t="n"/>
+      <c r="H28" s="49" t="n"/>
+      <c r="I28" s="49" t="n"/>
+      <c r="J28" s="49" t="n"/>
+      <c r="K28" s="49" t="n"/>
+      <c r="L28" s="49" t="n"/>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="49" t="n"/>
+      <c r="B29" s="53" t="inlineStr">
         <is>
           <t>VM5</t>
         </is>
       </c>
-      <c r="C30" s="45" t="inlineStr">
+      <c r="C29" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D30" s="45" t="n">
+      <c r="D29" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="45" t="inlineStr">
+      <c r="E29" s="53" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="F30" s="45" t="n"/>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="46" t="inlineStr">
+      <c r="F29" s="53" t="n"/>
+      <c r="G29" s="49" t="n"/>
+      <c r="H29" s="49" t="n"/>
+      <c r="I29" s="49" t="n"/>
+      <c r="J29" s="49" t="n"/>
+      <c r="K29" s="49" t="n"/>
+      <c r="L29" s="49" t="n"/>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="49" t="n"/>
+      <c r="B30" s="54" t="inlineStr">
         <is>
           <t>VM6</t>
         </is>
       </c>
-      <c r="C31" s="46" t="inlineStr">
+      <c r="C30" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D31" s="46" t="n">
+      <c r="D30" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E31" s="46" t="inlineStr">
+      <c r="E30" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F31" s="46" t="inlineStr">
+      <c r="F30" s="54" t="inlineStr">
         <is>
           <t>NS language; sig language</t>
         </is>
       </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="45" t="inlineStr">
+      <c r="G30" s="49" t="n"/>
+      <c r="H30" s="49" t="n"/>
+      <c r="I30" s="49" t="n"/>
+      <c r="J30" s="49" t="n"/>
+      <c r="K30" s="49" t="n"/>
+      <c r="L30" s="49" t="n"/>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="49" t="n"/>
+      <c r="B31" s="53" t="inlineStr">
         <is>
           <t>VM7</t>
         </is>
       </c>
-      <c r="C32" s="45" t="inlineStr">
+      <c r="C31" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D32" s="45" t="n">
+      <c r="D31" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="45" t="inlineStr">
+      <c r="E31" s="53" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F32" s="45" t="inlineStr">
+      <c r="F31" s="53" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="46" t="inlineStr">
+      <c r="G31" s="49" t="n"/>
+      <c r="H31" s="49" t="n"/>
+      <c r="I31" s="49" t="n"/>
+      <c r="J31" s="49" t="n"/>
+      <c r="K31" s="49" t="n"/>
+      <c r="L31" s="49" t="n"/>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="49" t="n"/>
+      <c r="B32" s="54" t="inlineStr">
         <is>
           <t>VM8</t>
         </is>
       </c>
-      <c r="C33" s="46" t="inlineStr">
+      <c r="C32" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D33" s="46" t="n">
+      <c r="D32" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="46" t="inlineStr">
+      <c r="E32" s="54" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="F33" s="46" t="n"/>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="45" t="inlineStr">
+      <c r="F32" s="54" t="n"/>
+      <c r="G32" s="49" t="n"/>
+      <c r="H32" s="49" t="n"/>
+      <c r="I32" s="49" t="n"/>
+      <c r="J32" s="49" t="n"/>
+      <c r="K32" s="49" t="n"/>
+      <c r="L32" s="49" t="n"/>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="49" t="n"/>
+      <c r="B33" s="53" t="inlineStr">
         <is>
           <t>VM9</t>
         </is>
       </c>
-      <c r="C34" s="45" t="inlineStr">
+      <c r="C33" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D34" s="45" t="n">
+      <c r="D33" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="45" t="inlineStr">
+      <c r="E33" s="53" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F34" s="45" t="inlineStr">
+      <c r="F33" s="53" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="B35" s="46" t="inlineStr">
+      <c r="G33" s="49" t="n"/>
+      <c r="H33" s="49" t="n"/>
+      <c r="I33" s="49" t="n"/>
+      <c r="J33" s="49" t="n"/>
+      <c r="K33" s="49" t="n"/>
+      <c r="L33" s="49" t="n"/>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="49" t="n"/>
+      <c r="B34" s="54" t="inlineStr">
         <is>
           <t>VM10</t>
         </is>
       </c>
-      <c r="C35" s="46" t="inlineStr">
+      <c r="C34" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D35" s="46" t="n">
+      <c r="D34" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="46" t="inlineStr">
+      <c r="E34" s="54" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F35" s="46" t="inlineStr">
+      <c r="F34" s="54" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="45" t="inlineStr">
+      <c r="G34" s="49" t="n"/>
+      <c r="H34" s="49" t="n"/>
+      <c r="I34" s="49" t="n"/>
+      <c r="J34" s="49" t="n"/>
+      <c r="K34" s="49" t="n"/>
+      <c r="L34" s="49" t="n"/>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="49" t="n"/>
+      <c r="B35" s="53" t="inlineStr">
         <is>
           <t>VM11</t>
         </is>
       </c>
-      <c r="C36" s="45" t="inlineStr">
+      <c r="C35" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D36" s="45" t="n">
+      <c r="D35" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E36" s="45" t="inlineStr">
+      <c r="E35" s="53" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F36" s="45" t="n"/>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="B37" s="46" t="inlineStr">
+      <c r="F35" s="53" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="49" t="n"/>
+      <c r="I35" s="49" t="n"/>
+      <c r="J35" s="49" t="n"/>
+      <c r="K35" s="49" t="n"/>
+      <c r="L35" s="49" t="n"/>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="49" t="n"/>
+      <c r="B36" s="54" t="inlineStr">
         <is>
           <t>VM12</t>
         </is>
       </c>
-      <c r="C37" s="46" t="inlineStr">
+      <c r="C36" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D37" s="46" t="n">
+      <c r="D36" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="E37" s="46" t="inlineStr">
+      <c r="E36" s="54" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F37" s="46" t="inlineStr">
+      <c r="F36" s="54" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-    </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="B38" s="45" t="inlineStr">
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="49" t="n"/>
+      <c r="I36" s="49" t="n"/>
+      <c r="J36" s="49" t="n"/>
+      <c r="K36" s="49" t="n"/>
+      <c r="L36" s="49" t="n"/>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="49" t="n"/>
+      <c r="B37" s="53" t="inlineStr">
         <is>
           <t>VM13</t>
         </is>
       </c>
-      <c r="C38" s="45" t="inlineStr">
+      <c r="C37" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D38" s="45" t="n">
+      <c r="D37" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E38" s="45" t="inlineStr">
+      <c r="E37" s="53" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F38" s="45" t="inlineStr">
+      <c r="F37" s="53" t="inlineStr">
         <is>
           <t>sig language</t>
         </is>
       </c>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="46" t="inlineStr">
+      <c r="G37" s="49" t="n"/>
+      <c r="H37" s="49" t="n"/>
+      <c r="I37" s="49" t="n"/>
+      <c r="J37" s="49" t="n"/>
+      <c r="K37" s="49" t="n"/>
+      <c r="L37" s="49" t="n"/>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="49" t="n"/>
+      <c r="B38" s="54" t="inlineStr">
         <is>
           <t>VM14</t>
         </is>
       </c>
-      <c r="C39" s="46" t="inlineStr">
+      <c r="C38" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D39" s="46" t="n">
+      <c r="D38" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E39" s="46" t="inlineStr">
+      <c r="E38" s="54" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="F39" s="46" t="n"/>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="B40" s="45" t="inlineStr">
+      <c r="F38" s="54" t="n"/>
+      <c r="G38" s="49" t="n"/>
+      <c r="H38" s="49" t="n"/>
+      <c r="I38" s="49" t="n"/>
+      <c r="J38" s="49" t="n"/>
+      <c r="K38" s="49" t="n"/>
+      <c r="L38" s="49" t="n"/>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="49" t="n"/>
+      <c r="B39" s="53" t="inlineStr">
         <is>
           <t>VM15</t>
         </is>
       </c>
-      <c r="C40" s="45" t="inlineStr">
+      <c r="C39" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D40" s="45" t="n">
+      <c r="D39" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E40" s="45" t="inlineStr">
+      <c r="E39" s="53" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="F40" s="45" t="n"/>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="B41" s="46" t="inlineStr">
+      <c r="F39" s="53" t="n"/>
+      <c r="G39" s="49" t="n"/>
+      <c r="H39" s="49" t="n"/>
+      <c r="I39" s="49" t="n"/>
+      <c r="J39" s="49" t="n"/>
+      <c r="K39" s="49" t="n"/>
+      <c r="L39" s="49" t="n"/>
+    </row>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="49" t="n"/>
+      <c r="B40" s="54" t="inlineStr">
         <is>
           <t>VM16</t>
         </is>
       </c>
-      <c r="C41" s="46" t="inlineStr">
+      <c r="C40" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D41" s="46" t="n">
+      <c r="D40" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E41" s="46" t="inlineStr">
+      <c r="E40" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F41" s="46" t="inlineStr">
+      <c r="F40" s="54" t="inlineStr">
         <is>
           <t>NS language; sig language</t>
         </is>
       </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="B42" s="45" t="inlineStr">
+      <c r="G40" s="49" t="n"/>
+      <c r="H40" s="49" t="n"/>
+      <c r="I40" s="49" t="n"/>
+      <c r="J40" s="49" t="n"/>
+      <c r="K40" s="49" t="n"/>
+      <c r="L40" s="49" t="n"/>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="49" t="n"/>
+      <c r="B41" s="53" t="inlineStr">
         <is>
           <t>VM17</t>
         </is>
       </c>
-      <c r="C42" s="45" t="inlineStr">
+      <c r="C41" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D42" s="45" t="n">
+      <c r="D41" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E42" s="45" t="inlineStr">
+      <c r="E41" s="53" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F42" s="45" t="inlineStr">
+      <c r="F41" s="53" t="inlineStr">
         <is>
           <t>sig language</t>
         </is>
       </c>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="B43" s="46" t="inlineStr">
+      <c r="G41" s="49" t="n"/>
+      <c r="H41" s="49" t="n"/>
+      <c r="I41" s="49" t="n"/>
+      <c r="J41" s="49" t="n"/>
+      <c r="K41" s="49" t="n"/>
+      <c r="L41" s="49" t="n"/>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="49" t="n"/>
+      <c r="B42" s="54" t="inlineStr">
         <is>
           <t>VM18</t>
         </is>
       </c>
-      <c r="C43" s="46" t="inlineStr">
+      <c r="C42" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D43" s="46" t="n">
+      <c r="D42" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E43" s="46" t="inlineStr">
+      <c r="E42" s="54" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F43" s="46" t="inlineStr">
+      <c r="F42" s="54" t="inlineStr">
         <is>
           <t>sig language</t>
         </is>
       </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="B44" s="45" t="inlineStr">
+      <c r="G42" s="49" t="n"/>
+      <c r="H42" s="49" t="n"/>
+      <c r="I42" s="49" t="n"/>
+      <c r="J42" s="49" t="n"/>
+      <c r="K42" s="49" t="n"/>
+      <c r="L42" s="49" t="n"/>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="49" t="n"/>
+      <c r="B43" s="53" t="inlineStr">
         <is>
           <t>VM19</t>
         </is>
       </c>
-      <c r="C44" s="45" t="inlineStr">
+      <c r="C43" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D44" s="45" t="n">
+      <c r="D43" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E44" s="45" t="inlineStr">
+      <c r="E43" s="53" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F44" s="45" t="n"/>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="B45" s="46" t="inlineStr">
+      <c r="F43" s="53" t="n"/>
+      <c r="G43" s="49" t="n"/>
+      <c r="H43" s="49" t="n"/>
+      <c r="I43" s="49" t="n"/>
+      <c r="J43" s="49" t="n"/>
+      <c r="K43" s="49" t="n"/>
+      <c r="L43" s="49" t="n"/>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="49" t="n"/>
+      <c r="B44" s="54" t="inlineStr">
         <is>
           <t>VM20</t>
         </is>
       </c>
-      <c r="C45" s="46" t="inlineStr">
+      <c r="C44" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D45" s="46" t="n">
+      <c r="D44" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E45" s="46" t="inlineStr">
+      <c r="E44" s="54" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F45" s="46" t="inlineStr">
+      <c r="F44" s="54" t="inlineStr">
         <is>
           <t>sig language</t>
         </is>
       </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="B46" s="45" t="inlineStr">
+      <c r="G44" s="49" t="n"/>
+      <c r="H44" s="49" t="n"/>
+      <c r="I44" s="49" t="n"/>
+      <c r="J44" s="49" t="n"/>
+      <c r="K44" s="49" t="n"/>
+      <c r="L44" s="49" t="n"/>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="49" t="n"/>
+      <c r="B45" s="53" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="C46" s="45" t="inlineStr">
+      <c r="C45" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D46" s="45" t="n">
+      <c r="D45" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="E46" s="45" t="inlineStr">
+      <c r="E45" s="53" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F46" s="45" t="inlineStr">
+      <c r="F45" s="53" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="B47" s="46" t="inlineStr">
+      <c r="G45" s="49" t="n"/>
+      <c r="H45" s="49" t="n"/>
+      <c r="I45" s="49" t="n"/>
+      <c r="J45" s="49" t="n"/>
+      <c r="K45" s="49" t="n"/>
+      <c r="L45" s="49" t="n"/>
+    </row>
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="49" t="n"/>
+      <c r="B46" s="54" t="inlineStr">
         <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="C47" s="46" t="inlineStr">
+      <c r="C46" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D47" s="46" t="n">
+      <c r="D46" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E47" s="46" t="inlineStr">
+      <c r="E46" s="54" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F47" s="46" t="inlineStr">
+      <c r="F46" s="54" t="inlineStr">
         <is>
           <t>no zone of inhibition / did not possess</t>
         </is>
       </c>
-    </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="B48" s="45" t="inlineStr">
+      <c r="G46" s="49" t="n"/>
+      <c r="H46" s="49" t="n"/>
+      <c r="I46" s="49" t="n"/>
+      <c r="J46" s="49" t="n"/>
+      <c r="K46" s="49" t="n"/>
+      <c r="L46" s="49" t="n"/>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="49" t="n"/>
+      <c r="B47" s="53" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
-      <c r="C48" s="45" t="inlineStr">
+      <c r="C47" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D48" s="45" t="n">
+      <c r="D47" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E48" s="45" t="inlineStr">
+      <c r="E47" s="53" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F48" s="45" t="n"/>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="B49" s="46" t="inlineStr">
+      <c r="F47" s="53" t="n"/>
+      <c r="G47" s="49" t="n"/>
+      <c r="H47" s="49" t="n"/>
+      <c r="I47" s="49" t="n"/>
+      <c r="J47" s="49" t="n"/>
+      <c r="K47" s="49" t="n"/>
+      <c r="L47" s="49" t="n"/>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="49" t="n"/>
+      <c r="B48" s="54" t="inlineStr">
         <is>
           <t>B4</t>
         </is>
       </c>
-      <c r="C49" s="46" t="inlineStr">
+      <c r="C48" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D49" s="46" t="n">
+      <c r="D48" s="54" t="n">
         <v>3</v>
       </c>
-      <c r="E49" s="46" t="inlineStr">
+      <c r="E48" s="54" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="F49" s="46" t="n"/>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="B50" s="45" t="inlineStr">
+      <c r="F48" s="54" t="n"/>
+      <c r="G48" s="49" t="n"/>
+      <c r="H48" s="49" t="n"/>
+      <c r="I48" s="49" t="n"/>
+      <c r="J48" s="49" t="n"/>
+      <c r="K48" s="49" t="n"/>
+      <c r="L48" s="49" t="n"/>
+    </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="49" t="n"/>
+      <c r="B49" s="53" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="C50" s="45" t="inlineStr">
+      <c r="C49" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D50" s="45" t="n">
+      <c r="D49" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E50" s="45" t="inlineStr">
+      <c r="E49" s="53" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F50" s="45" t="inlineStr">
+      <c r="F49" s="53" t="inlineStr">
         <is>
           <t>NS language; sig language</t>
         </is>
       </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="B51" s="46" t="inlineStr">
+      <c r="G49" s="49" t="n"/>
+      <c r="H49" s="49" t="n"/>
+      <c r="I49" s="49" t="n"/>
+      <c r="J49" s="49" t="n"/>
+      <c r="K49" s="49" t="n"/>
+      <c r="L49" s="49" t="n"/>
+    </row>
+    <row r="50" ht="28" customHeight="1">
+      <c r="A50" s="49" t="n"/>
+      <c r="B50" s="54" t="inlineStr">
         <is>
           <t>B6</t>
         </is>
       </c>
-      <c r="C51" s="46" t="inlineStr">
+      <c r="C50" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D51" s="46" t="n">
+      <c r="D50" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="E51" s="46" t="inlineStr">
+      <c r="E50" s="54" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F51" s="46" t="n"/>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="B52" s="45" t="inlineStr">
+      <c r="F50" s="54" t="n"/>
+      <c r="G50" s="49" t="n"/>
+      <c r="H50" s="49" t="n"/>
+      <c r="I50" s="49" t="n"/>
+      <c r="J50" s="49" t="n"/>
+      <c r="K50" s="49" t="n"/>
+      <c r="L50" s="49" t="n"/>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="49" t="n"/>
+      <c r="B51" s="53" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="C52" s="45" t="inlineStr">
+      <c r="C51" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D52" s="45" t="n">
+      <c r="D51" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="E52" s="45" t="inlineStr">
+      <c r="E51" s="53" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="F52" s="45" t="n"/>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="B53" s="46" t="inlineStr">
+      <c r="F51" s="53" t="n"/>
+      <c r="G51" s="49" t="n"/>
+      <c r="H51" s="49" t="n"/>
+      <c r="I51" s="49" t="n"/>
+      <c r="J51" s="49" t="n"/>
+      <c r="K51" s="49" t="n"/>
+      <c r="L51" s="49" t="n"/>
+    </row>
+    <row r="52" ht="28" customHeight="1">
+      <c r="A52" s="49" t="n"/>
+      <c r="B52" s="54" t="inlineStr">
         <is>
           <t>B8</t>
         </is>
       </c>
-      <c r="C53" s="46" t="inlineStr">
+      <c r="C52" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D53" s="46" t="n">
+      <c r="D52" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E53" s="46" t="inlineStr">
+      <c r="E52" s="54" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F53" s="46" t="inlineStr">
+      <c r="F52" s="54" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="B54" s="45" t="inlineStr">
+      <c r="G52" s="49" t="n"/>
+      <c r="H52" s="49" t="n"/>
+      <c r="I52" s="49" t="n"/>
+      <c r="J52" s="49" t="n"/>
+      <c r="K52" s="49" t="n"/>
+      <c r="L52" s="49" t="n"/>
+    </row>
+    <row r="53" ht="28" customHeight="1">
+      <c r="A53" s="49" t="n"/>
+      <c r="B53" s="53" t="inlineStr">
         <is>
           <t>B9</t>
         </is>
       </c>
-      <c r="C54" s="45" t="inlineStr">
+      <c r="C53" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D54" s="45" t="n">
+      <c r="D53" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E54" s="45" t="inlineStr">
+      <c r="E53" s="53" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="F54" s="45" t="inlineStr">
+      <c r="F53" s="53" t="inlineStr">
         <is>
           <t>NS language</t>
         </is>
       </c>
-    </row>
-    <row r="55" ht="22" customHeight="1">
-      <c r="B55" s="46" t="inlineStr">
+      <c r="G53" s="49" t="n"/>
+      <c r="H53" s="49" t="n"/>
+      <c r="I53" s="49" t="n"/>
+      <c r="J53" s="49" t="n"/>
+      <c r="K53" s="49" t="n"/>
+      <c r="L53" s="49" t="n"/>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="49" t="n"/>
+      <c r="B54" s="54" t="inlineStr">
         <is>
           <t>B10</t>
         </is>
       </c>
-      <c r="C55" s="46" t="inlineStr">
+      <c r="C54" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D55" s="46" t="n">
+      <c r="D54" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="E55" s="46" t="inlineStr">
+      <c r="E54" s="54" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="F55" s="46" t="n"/>
-    </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="B56" s="45" t="inlineStr">
+      <c r="F54" s="54" t="n"/>
+      <c r="G54" s="49" t="n"/>
+      <c r="H54" s="49" t="n"/>
+      <c r="I54" s="49" t="n"/>
+      <c r="J54" s="49" t="n"/>
+      <c r="K54" s="49" t="n"/>
+      <c r="L54" s="49" t="n"/>
+    </row>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="49" t="n"/>
+      <c r="B55" s="53" t="inlineStr">
         <is>
           <t>B11</t>
         </is>
       </c>
-      <c r="C56" s="45" t="inlineStr">
+      <c r="C55" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D56" s="45" t="n">
+      <c r="D55" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E56" s="45" t="inlineStr">
+      <c r="E55" s="53" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F56" s="45" t="inlineStr">
+      <c r="F55" s="53" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-    </row>
-    <row r="57" ht="22" customHeight="1">
-      <c r="B57" s="46" t="inlineStr">
+      <c r="G55" s="49" t="n"/>
+      <c r="H55" s="49" t="n"/>
+      <c r="I55" s="49" t="n"/>
+      <c r="J55" s="49" t="n"/>
+      <c r="K55" s="49" t="n"/>
+      <c r="L55" s="49" t="n"/>
+    </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="49" t="n"/>
+      <c r="B56" s="54" t="inlineStr">
         <is>
           <t>B12</t>
         </is>
       </c>
-      <c r="C57" s="46" t="inlineStr">
+      <c r="C56" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D57" s="46" t="n">
+      <c r="D56" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="E57" s="46" t="inlineStr">
+      <c r="E56" s="54" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="F57" s="46" t="n"/>
-    </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="B58" s="45" t="inlineStr">
+      <c r="F56" s="54" t="n"/>
+      <c r="G56" s="49" t="n"/>
+      <c r="H56" s="49" t="n"/>
+      <c r="I56" s="49" t="n"/>
+      <c r="J56" s="49" t="n"/>
+      <c r="K56" s="49" t="n"/>
+      <c r="L56" s="49" t="n"/>
+    </row>
+    <row r="57" ht="28" customHeight="1">
+      <c r="A57" s="49" t="n"/>
+      <c r="B57" s="53" t="inlineStr">
         <is>
           <t>B13</t>
         </is>
       </c>
-      <c r="C58" s="45" t="inlineStr">
+      <c r="C57" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D58" s="45" t="n">
+      <c r="D57" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E58" s="45" t="inlineStr">
+      <c r="E57" s="53" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="F58" s="45" t="n"/>
-    </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="B59" s="46" t="inlineStr">
+      <c r="F57" s="53" t="n"/>
+      <c r="G57" s="49" t="n"/>
+      <c r="H57" s="49" t="n"/>
+      <c r="I57" s="49" t="n"/>
+      <c r="J57" s="49" t="n"/>
+      <c r="K57" s="49" t="n"/>
+      <c r="L57" s="49" t="n"/>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="49" t="n"/>
+      <c r="B58" s="54" t="inlineStr">
         <is>
           <t>B14</t>
         </is>
       </c>
-      <c r="C59" s="46" t="inlineStr">
+      <c r="C58" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D59" s="46" t="n">
+      <c r="D58" s="54" t="n">
         <v>3</v>
       </c>
-      <c r="E59" s="46" t="inlineStr">
+      <c r="E58" s="54" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="F59" s="46" t="n"/>
-    </row>
-    <row r="60" ht="22" customHeight="1">
-      <c r="B60" s="45" t="inlineStr">
+      <c r="F58" s="54" t="n"/>
+      <c r="G58" s="49" t="n"/>
+      <c r="H58" s="49" t="n"/>
+      <c r="I58" s="49" t="n"/>
+      <c r="J58" s="49" t="n"/>
+      <c r="K58" s="49" t="n"/>
+      <c r="L58" s="49" t="n"/>
+    </row>
+    <row r="59" ht="28" customHeight="1">
+      <c r="A59" s="49" t="n"/>
+      <c r="B59" s="53" t="inlineStr">
         <is>
           <t>B15</t>
         </is>
       </c>
-      <c r="C60" s="45" t="inlineStr">
+      <c r="C59" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D60" s="45" t="n">
+      <c r="D59" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="E60" s="45" t="inlineStr">
+      <c r="E59" s="53" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="F60" s="45" t="n"/>
-    </row>
-    <row r="61" ht="22" customHeight="1">
-      <c r="B61" s="46" t="inlineStr">
+      <c r="F59" s="53" t="n"/>
+      <c r="G59" s="49" t="n"/>
+      <c r="H59" s="49" t="n"/>
+      <c r="I59" s="49" t="n"/>
+      <c r="J59" s="49" t="n"/>
+      <c r="K59" s="49" t="n"/>
+      <c r="L59" s="49" t="n"/>
+    </row>
+    <row r="60" ht="28" customHeight="1">
+      <c r="A60" s="49" t="n"/>
+      <c r="B60" s="54" t="inlineStr">
         <is>
           <t>B16</t>
         </is>
       </c>
-      <c r="C61" s="46" t="inlineStr">
+      <c r="C60" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D61" s="46" t="n">
+      <c r="D60" s="54" t="n">
         <v>5</v>
       </c>
-      <c r="E61" s="46" t="inlineStr">
+      <c r="E60" s="54" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F61" s="46" t="inlineStr">
+      <c r="F60" s="54" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-    </row>
-    <row r="62" ht="22" customHeight="1">
-      <c r="B62" s="45" t="inlineStr">
+      <c r="G60" s="49" t="n"/>
+      <c r="H60" s="49" t="n"/>
+      <c r="I60" s="49" t="n"/>
+      <c r="J60" s="49" t="n"/>
+      <c r="K60" s="49" t="n"/>
+      <c r="L60" s="49" t="n"/>
+    </row>
+    <row r="61" ht="28" customHeight="1">
+      <c r="A61" s="49" t="n"/>
+      <c r="B61" s="53" t="inlineStr">
         <is>
           <t>B17</t>
         </is>
       </c>
-      <c r="C62" s="45" t="inlineStr">
+      <c r="C61" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D62" s="45" t="n">
+      <c r="D61" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="E62" s="45" t="inlineStr">
+      <c r="E61" s="53" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F62" s="45" t="n"/>
-    </row>
-    <row r="63" ht="22" customHeight="1">
-      <c r="B63" s="46" t="inlineStr">
+      <c r="F61" s="53" t="n"/>
+      <c r="G61" s="49" t="n"/>
+      <c r="H61" s="49" t="n"/>
+      <c r="I61" s="49" t="n"/>
+      <c r="J61" s="49" t="n"/>
+      <c r="K61" s="49" t="n"/>
+      <c r="L61" s="49" t="n"/>
+    </row>
+    <row r="62" ht="28" customHeight="1">
+      <c r="A62" s="49" t="n"/>
+      <c r="B62" s="54" t="inlineStr">
         <is>
           <t>B18</t>
         </is>
       </c>
-      <c r="C63" s="46" t="inlineStr">
+      <c r="C62" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D63" s="46" t="n">
+      <c r="D62" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="E63" s="46" t="inlineStr">
+      <c r="E62" s="54" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F63" s="46" t="inlineStr">
+      <c r="F62" s="54" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-    </row>
-    <row r="64" ht="22" customHeight="1">
-      <c r="B64" s="45" t="inlineStr">
+      <c r="G62" s="49" t="n"/>
+      <c r="H62" s="49" t="n"/>
+      <c r="I62" s="49" t="n"/>
+      <c r="J62" s="49" t="n"/>
+      <c r="K62" s="49" t="n"/>
+      <c r="L62" s="49" t="n"/>
+    </row>
+    <row r="63" ht="28" customHeight="1">
+      <c r="A63" s="49" t="n"/>
+      <c r="B63" s="53" t="inlineStr">
         <is>
           <t>B19</t>
         </is>
       </c>
-      <c r="C64" s="45" t="inlineStr">
+      <c r="C63" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D64" s="45" t="n">
+      <c r="D63" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E64" s="45" t="inlineStr">
+      <c r="E63" s="53" t="inlineStr">
         <is>
           <t>Binary</t>
         </is>
       </c>
-      <c r="F64" s="45" t="n"/>
+      <c r="F63" s="53" t="n"/>
+      <c r="G63" s="49" t="n"/>
+      <c r="H63" s="49" t="n"/>
+      <c r="I63" s="49" t="n"/>
+      <c r="J63" s="49" t="n"/>
+      <c r="K63" s="49" t="n"/>
+      <c r="L63" s="49" t="n"/>
+    </row>
+    <row r="64" ht="28" customHeight="1">
+      <c r="A64" s="49" t="n"/>
+      <c r="B64" s="54" t="inlineStr">
+        <is>
+          <t>B20</t>
+        </is>
+      </c>
+      <c r="C64" s="54" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="D64" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="54" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="F64" s="54" t="inlineStr">
+        <is>
+          <t>NS language</t>
+        </is>
+      </c>
+      <c r="G64" s="49" t="n"/>
+      <c r="H64" s="49" t="n"/>
+      <c r="I64" s="49" t="n"/>
+      <c r="J64" s="49" t="n"/>
+      <c r="K64" s="49" t="n"/>
+      <c r="L64" s="49" t="n"/>
     </row>
     <row r="65" ht="22" customHeight="1">
-      <c r="B65" s="46" t="inlineStr">
-        <is>
-          <t>B20</t>
-        </is>
-      </c>
-      <c r="C65" s="46" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="D65" s="46" t="n">
-        <v>1</v>
-      </c>
-      <c r="E65" s="46" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="F65" s="46" t="inlineStr">
-        <is>
-          <t>NS language</t>
-        </is>
-      </c>
+      <c r="A65" s="49" t="n"/>
+      <c r="B65" s="49" t="n"/>
+      <c r="C65" s="49" t="n"/>
+      <c r="D65" s="49" t="n"/>
+      <c r="E65" s="49" t="n"/>
+      <c r="F65" s="49" t="n"/>
+      <c r="G65" s="49" t="n"/>
+      <c r="H65" s="49" t="n"/>
+      <c r="I65" s="49" t="n"/>
+      <c r="J65" s="49" t="n"/>
+      <c r="K65" s="49" t="n"/>
+      <c r="L65" s="49" t="n"/>
     </row>
     <row r="66" ht="32" customHeight="1">
-      <c r="B66" s="46" t="n"/>
-      <c r="C66" s="46" t="n"/>
-      <c r="D66" s="46" t="n"/>
-      <c r="E66" s="46" t="n"/>
-      <c r="F66" s="46" t="n"/>
+      <c r="A66" s="49" t="n"/>
+      <c r="B66" s="49" t="n"/>
+      <c r="C66" s="49" t="n"/>
+      <c r="D66" s="49" t="n"/>
+      <c r="E66" s="49" t="n"/>
+      <c r="F66" s="49" t="n"/>
+      <c r="G66" s="49" t="n"/>
+      <c r="H66" s="49" t="n"/>
+      <c r="I66" s="49" t="n"/>
+      <c r="J66" s="49" t="n"/>
+      <c r="K66" s="49" t="n"/>
+      <c r="L66" s="49" t="n"/>
     </row>
     <row r="67" ht="32" customHeight="1">
-      <c r="B67" s="46" t="n"/>
-      <c r="C67" s="46" t="n"/>
-      <c r="D67" s="46" t="n"/>
-      <c r="E67" s="46" t="n"/>
-      <c r="F67" s="46" t="n"/>
+      <c r="A67" s="49" t="n"/>
+      <c r="B67" s="49" t="n"/>
+      <c r="C67" s="49" t="n"/>
+      <c r="D67" s="49" t="n"/>
+      <c r="E67" s="49" t="n"/>
+      <c r="F67" s="49" t="n"/>
+      <c r="G67" s="49" t="n"/>
+      <c r="H67" s="49" t="n"/>
+      <c r="I67" s="49" t="n"/>
+      <c r="J67" s="49" t="n"/>
+      <c r="K67" s="49" t="n"/>
+      <c r="L67" s="49" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10588,7 +11124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I26"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -10602,943 +11138,1137 @@
     <col width="55" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="49" t="n"/>
+      <c r="B1" s="49" t="n"/>
+      <c r="C1" s="49" t="n"/>
+      <c r="D1" s="49" t="n"/>
+      <c r="E1" s="49" t="n"/>
+      <c r="F1" s="49" t="n"/>
+      <c r="G1" s="49" t="n"/>
+      <c r="H1" s="49" t="n"/>
+      <c r="I1" s="49" t="n"/>
+      <c r="J1" s="49" t="n"/>
+      <c r="K1" s="49" t="n"/>
+      <c r="L1" s="49" t="n"/>
+    </row>
     <row r="2">
-      <c r="B2" s="17" t="inlineStr">
+      <c r="A2" s="49" t="n"/>
+      <c r="B2" s="50" t="inlineStr">
         <is>
           <t>P and DO Functions — Scan Log (Non-Hedge Inventory)</t>
         </is>
       </c>
+      <c r="C2" s="49" t="n"/>
+      <c r="D2" s="49" t="n"/>
+      <c r="E2" s="49" t="n"/>
+      <c r="F2" s="49" t="n"/>
+      <c r="G2" s="49" t="n"/>
+      <c r="H2" s="49" t="n"/>
+      <c r="I2" s="49" t="n"/>
+      <c r="J2" s="49" t="n"/>
+      <c r="K2" s="49" t="n"/>
+      <c r="L2" s="49" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="43" t="inlineStr">
+      <c r="A3" s="49" t="n"/>
+      <c r="B3" s="51" t="inlineStr">
         <is>
           <t>Discourse-organization connectors and politeness scan across 60 abstracts. Hedge? = N for all. Not counted in Layer 1/2 totals.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="B5" s="44" t="inlineStr">
+      <c r="C3" s="49" t="n"/>
+      <c r="D3" s="49" t="n"/>
+      <c r="E3" s="49" t="n"/>
+      <c r="F3" s="49" t="n"/>
+      <c r="G3" s="49" t="n"/>
+      <c r="H3" s="49" t="n"/>
+      <c r="I3" s="49" t="n"/>
+      <c r="J3" s="49" t="n"/>
+      <c r="K3" s="49" t="n"/>
+      <c r="L3" s="49" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="49" t="n"/>
+      <c r="B4" s="52" t="inlineStr">
         <is>
           <t>Abstract ID</t>
         </is>
       </c>
-      <c r="C5" s="44" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>Discipline</t>
         </is>
       </c>
-      <c r="D5" s="44" t="inlineStr">
+      <c r="D4" s="52" t="inlineStr">
         <is>
           <t>Phrase / Token</t>
         </is>
       </c>
-      <c r="E5" s="44" t="inlineStr">
+      <c r="E4" s="52" t="inlineStr">
         <is>
           <t>Context (short)</t>
         </is>
       </c>
-      <c r="F5" s="44" t="inlineStr">
+      <c r="F4" s="52" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="G5" s="44" t="inlineStr">
+      <c r="G4" s="52" t="inlineStr">
         <is>
           <t>Hedge?</t>
         </is>
       </c>
-      <c r="H5" s="44" t="inlineStr">
+      <c r="H4" s="52" t="inlineStr">
         <is>
           <t>Ambiguous</t>
         </is>
       </c>
-      <c r="I5" s="44" t="inlineStr">
+      <c r="I4" s="52" t="inlineStr">
         <is>
           <t>Reasoning</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="B6" s="45" t="inlineStr">
+      <c r="J4" s="49" t="n"/>
+      <c r="K4" s="49" t="n"/>
+      <c r="L4" s="49" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="49" t="n"/>
+      <c r="B5" s="53" t="inlineStr">
         <is>
           <t>B6</t>
         </is>
       </c>
-      <c r="C6" s="45" t="inlineStr">
+      <c r="C5" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D6" s="45" t="inlineStr">
+      <c r="D5" s="53" t="inlineStr">
         <is>
           <t>Thus / Therefore</t>
         </is>
       </c>
-      <c r="E6" s="45" t="inlineStr">
+      <c r="E5" s="53" t="inlineStr">
         <is>
           <t>Thus, in the optimization process...; Therefore, further research will...</t>
         </is>
       </c>
-      <c r="F6" s="45" t="inlineStr">
+      <c r="F5" s="53" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G6" s="45" t="inlineStr">
+      <c r="G5" s="53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H6" s="45" t="inlineStr">
+      <c r="H5" s="53" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I6" s="45" t="inlineStr">
+      <c r="I5" s="53" t="inlineStr">
         <is>
           <t>Move connectors (problem→method; limit→future work). Not epistemic hedges.</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="46" t="inlineStr">
+      <c r="J5" s="49" t="n"/>
+      <c r="K5" s="49" t="n"/>
+      <c r="L5" s="49" t="n"/>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="49" t="n"/>
+      <c r="B6" s="54" t="inlineStr">
         <is>
           <t>B7</t>
         </is>
       </c>
-      <c r="C7" s="46" t="inlineStr">
+      <c r="C6" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D7" s="46" t="inlineStr">
+      <c r="D6" s="54" t="inlineStr">
         <is>
           <t>Hence / thus</t>
         </is>
       </c>
-      <c r="E7" s="46" t="inlineStr">
+      <c r="E6" s="54" t="inlineStr">
         <is>
           <t>Hence, the biosynthesis is feasible; thus making a remarkable choice; thus demonstrating...</t>
         </is>
       </c>
-      <c r="F7" s="46" t="inlineStr">
+      <c r="F6" s="54" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G7" s="46" t="inlineStr">
+      <c r="G6" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H7" s="46" t="inlineStr">
+      <c r="H6" s="54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I7" s="46" t="inlineStr">
+      <c r="I6" s="54" t="inlineStr">
         <is>
           <t>Claim-sequence connectors. Hedge if any is separate (may).</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="B8" s="45" t="inlineStr">
+      <c r="J6" s="49" t="n"/>
+      <c r="K6" s="49" t="n"/>
+      <c r="L6" s="49" t="n"/>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="49" t="n"/>
+      <c r="B7" s="53" t="inlineStr">
         <is>
           <t>B10</t>
         </is>
       </c>
-      <c r="C8" s="45" t="inlineStr">
+      <c r="C7" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D8" s="45" t="inlineStr">
+      <c r="D7" s="53" t="inlineStr">
         <is>
           <t>Thus</t>
         </is>
       </c>
-      <c r="E8" s="45" t="inlineStr">
+      <c r="E7" s="53" t="inlineStr">
         <is>
           <t>Thus, the researcher provided a policy proposal...</t>
         </is>
       </c>
-      <c r="F8" s="45" t="inlineStr">
+      <c r="F7" s="53" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G8" s="45" t="inlineStr">
+      <c r="G7" s="53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H8" s="45" t="inlineStr">
+      <c r="H7" s="53" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I8" s="45" t="inlineStr">
+      <c r="I7" s="53" t="inlineStr">
         <is>
           <t>Results→recommendation connector.</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="46" t="inlineStr">
+      <c r="J7" s="49" t="n"/>
+      <c r="K7" s="49" t="n"/>
+      <c r="L7" s="49" t="n"/>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="49" t="n"/>
+      <c r="B8" s="54" t="inlineStr">
         <is>
           <t>B11</t>
         </is>
       </c>
-      <c r="C9" s="46" t="inlineStr">
+      <c r="C8" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D9" s="46" t="inlineStr">
+      <c r="D8" s="54" t="inlineStr">
         <is>
           <t>Hence</t>
         </is>
       </c>
-      <c r="E9" s="46" t="inlineStr">
+      <c r="E8" s="54" t="inlineStr">
         <is>
           <t>Hence, this study aimed to investigate...</t>
         </is>
       </c>
-      <c r="F9" s="46" t="inlineStr">
+      <c r="F8" s="54" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G9" s="46" t="inlineStr">
+      <c r="G8" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H9" s="46" t="inlineStr">
+      <c r="H8" s="54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I9" s="46" t="inlineStr">
+      <c r="I8" s="54" t="inlineStr">
         <is>
           <t>Background→aim connector.</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="B10" s="45" t="inlineStr">
+      <c r="J8" s="49" t="n"/>
+      <c r="K8" s="49" t="n"/>
+      <c r="L8" s="49" t="n"/>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="49" t="n"/>
+      <c r="B9" s="53" t="inlineStr">
         <is>
           <t>B12</t>
         </is>
       </c>
-      <c r="C10" s="45" t="inlineStr">
+      <c r="C9" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D10" s="45" t="inlineStr">
+      <c r="D9" s="53" t="inlineStr">
         <is>
           <t>Hence</t>
         </is>
       </c>
-      <c r="E10" s="45" t="inlineStr">
+      <c r="E9" s="53" t="inlineStr">
         <is>
           <t>Hence, LAB have emerged as a focal point...</t>
         </is>
       </c>
-      <c r="F10" s="45" t="inlineStr">
+      <c r="F9" s="53" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G10" s="45" t="inlineStr">
+      <c r="G9" s="53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H10" s="45" t="inlineStr">
+      <c r="H9" s="53" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I10" s="45" t="inlineStr">
+      <c r="I9" s="53" t="inlineStr">
         <is>
           <t>Problem→focus connector.</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="B11" s="46" t="inlineStr">
+      <c r="J9" s="49" t="n"/>
+      <c r="K9" s="49" t="n"/>
+      <c r="L9" s="49" t="n"/>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="49" t="n"/>
+      <c r="B10" s="54" t="inlineStr">
         <is>
           <t>B16</t>
         </is>
       </c>
-      <c r="C11" s="46" t="inlineStr">
+      <c r="C10" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D11" s="46" t="inlineStr">
+      <c r="D10" s="54" t="inlineStr">
         <is>
           <t>Thus / therefore</t>
         </is>
       </c>
-      <c r="E11" s="46" t="inlineStr">
+      <c r="E10" s="54" t="inlineStr">
         <is>
           <t>Thus, this study detected...; This study, therefore, underscores...</t>
         </is>
       </c>
-      <c r="F11" s="46" t="inlineStr">
+      <c r="F10" s="54" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G11" s="46" t="inlineStr">
+      <c r="G10" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H11" s="46" t="inlineStr">
+      <c r="H10" s="54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I11" s="46" t="inlineStr">
+      <c r="I10" s="54" t="inlineStr">
         <is>
           <t>Rationale→aim / findings→implication connectors.</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="B12" s="45" t="inlineStr">
+      <c r="J10" s="49" t="n"/>
+      <c r="K10" s="49" t="n"/>
+      <c r="L10" s="49" t="n"/>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="49" t="n"/>
+      <c r="B11" s="53" t="inlineStr">
         <is>
           <t>B19</t>
         </is>
       </c>
-      <c r="C12" s="45" t="inlineStr">
+      <c r="C11" s="53" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D12" s="45" t="inlineStr">
+      <c r="D11" s="53" t="inlineStr">
         <is>
           <t>Hence / Thus</t>
         </is>
       </c>
-      <c r="E12" s="45" t="inlineStr">
+      <c r="E11" s="53" t="inlineStr">
         <is>
           <t>Hence, sustainable planning should...; Thus, local government should...</t>
         </is>
       </c>
-      <c r="F12" s="45" t="inlineStr">
+      <c r="F11" s="53" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G12" s="45" t="inlineStr">
+      <c r="G11" s="53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H12" s="45" t="inlineStr">
+      <c r="H11" s="53" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I12" s="45" t="inlineStr">
+      <c r="I11" s="53" t="inlineStr">
         <is>
           <t>Problem/findings→recommendation connectors.</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="B13" s="46" t="inlineStr">
+      <c r="J11" s="49" t="n"/>
+      <c r="K11" s="49" t="n"/>
+      <c r="L11" s="49" t="n"/>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="49" t="n"/>
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>B20</t>
         </is>
       </c>
-      <c r="C13" s="46" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D13" s="46" t="inlineStr">
+      <c r="D12" s="54" t="inlineStr">
         <is>
           <t>Therefore / Hence</t>
         </is>
       </c>
-      <c r="E13" s="46" t="inlineStr">
+      <c r="E12" s="54" t="inlineStr">
         <is>
           <t>Therefore, this study aims...; Hence, the study aimed...</t>
         </is>
       </c>
-      <c r="F13" s="46" t="inlineStr">
+      <c r="F12" s="54" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G13" s="46" t="inlineStr">
+      <c r="G12" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H13" s="46" t="inlineStr">
+      <c r="H12" s="54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I13" s="46" t="inlineStr">
+      <c r="I12" s="54" t="inlineStr">
         <is>
           <t>Background→aim connectors.</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="B14" s="45" t="inlineStr">
+      <c r="J12" s="49" t="n"/>
+      <c r="K12" s="49" t="n"/>
+      <c r="L12" s="49" t="n"/>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="49" t="n"/>
+      <c r="B13" s="53" t="inlineStr">
         <is>
           <t>VM7</t>
         </is>
       </c>
-      <c r="C14" s="45" t="inlineStr">
+      <c r="C13" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D14" s="45" t="inlineStr">
+      <c r="D13" s="53" t="inlineStr">
         <is>
           <t>Thus</t>
         </is>
       </c>
-      <c r="E14" s="45" t="inlineStr">
+      <c r="E13" s="53" t="inlineStr">
         <is>
           <t>Thus, no significant association could be established</t>
         </is>
       </c>
-      <c r="F14" s="45" t="inlineStr">
+      <c r="F13" s="53" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G14" s="45" t="inlineStr">
+      <c r="G13" s="53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H14" s="45" t="inlineStr">
+      <c r="H13" s="53" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I14" s="45" t="inlineStr">
+      <c r="I13" s="53" t="inlineStr">
         <is>
           <t>Results→conclusion connector.</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="B15" s="46" t="inlineStr">
+      <c r="J13" s="49" t="n"/>
+      <c r="K13" s="49" t="n"/>
+      <c r="L13" s="49" t="n"/>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="49" t="n"/>
+      <c r="B14" s="54" t="inlineStr">
         <is>
           <t>VM9</t>
         </is>
       </c>
-      <c r="C15" s="46" t="inlineStr">
+      <c r="C14" s="54" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D15" s="46" t="inlineStr">
+      <c r="D14" s="54" t="inlineStr">
         <is>
           <t>hence</t>
         </is>
       </c>
-      <c r="E15" s="46" t="inlineStr">
+      <c r="E14" s="54" t="inlineStr">
         <is>
           <t>hence, all individual shrimps counted as one sample</t>
         </is>
       </c>
-      <c r="F15" s="46" t="inlineStr">
+      <c r="F14" s="54" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G15" s="46" t="inlineStr">
+      <c r="G14" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H15" s="46" t="inlineStr">
+      <c r="H14" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I15" s="46" t="inlineStr">
+      <c r="I14" s="54" t="inlineStr">
         <is>
           <t>Methods sequencing only.</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="B16" s="45" t="inlineStr">
+      <c r="J14" s="49" t="n"/>
+      <c r="K14" s="49" t="n"/>
+      <c r="L14" s="49" t="n"/>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="49" t="n"/>
+      <c r="B15" s="53" t="inlineStr">
         <is>
           <t>VM12</t>
         </is>
       </c>
-      <c r="C16" s="45" t="inlineStr">
+      <c r="C15" s="53" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D16" s="45" t="inlineStr">
+      <c r="D15" s="53" t="inlineStr">
         <is>
           <t>Hence</t>
         </is>
       </c>
-      <c r="E16" s="45" t="inlineStr">
+      <c r="E15" s="53" t="inlineStr">
         <is>
           <t>Hence, this study aimed to detect ASF virus...</t>
         </is>
       </c>
-      <c r="F16" s="45" t="inlineStr">
+      <c r="F15" s="53" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G16" s="45" t="inlineStr">
+      <c r="G15" s="53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H16" s="45" t="inlineStr">
+      <c r="H15" s="53" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I16" s="45" t="inlineStr">
+      <c r="I15" s="53" t="inlineStr">
         <is>
           <t>Background→aim connector.</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="B17" s="46" t="inlineStr">
+      <c r="J15" s="49" t="n"/>
+      <c r="K15" s="49" t="n"/>
+      <c r="L15" s="49" t="n"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="49" t="n"/>
+      <c r="B16" s="54" t="inlineStr">
         <is>
           <t>Acs5</t>
         </is>
       </c>
-      <c r="C17" s="46" t="inlineStr">
+      <c r="C16" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D17" s="46" t="inlineStr">
+      <c r="D16" s="54" t="inlineStr">
         <is>
           <t>Therefore</t>
         </is>
       </c>
-      <c r="E17" s="46" t="inlineStr">
+      <c r="E16" s="54" t="inlineStr">
         <is>
           <t>Therefore, the... (yield inference connector)</t>
         </is>
       </c>
-      <c r="F17" s="46" t="inlineStr">
+      <c r="F16" s="54" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G17" s="46" t="inlineStr">
+      <c r="G16" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H17" s="46" t="inlineStr">
+      <c r="H16" s="54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I17" s="46" t="inlineStr">
+      <c r="I16" s="54" t="inlineStr">
         <is>
           <t>Results→inference connector.</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="32" customHeight="1">
-      <c r="B18" s="45" t="inlineStr">
+      <c r="J16" s="49" t="n"/>
+      <c r="K16" s="49" t="n"/>
+      <c r="L16" s="49" t="n"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="49" t="n"/>
+      <c r="B17" s="53" t="inlineStr">
         <is>
           <t>Aas9</t>
         </is>
       </c>
-      <c r="C18" s="45" t="inlineStr">
+      <c r="C17" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D18" s="45" t="inlineStr">
+      <c r="D17" s="53" t="inlineStr">
         <is>
           <t>Therefore</t>
         </is>
       </c>
-      <c r="E18" s="45" t="inlineStr">
+      <c r="E17" s="53" t="inlineStr">
         <is>
           <t>Therefore, it is recommended for future researchers...</t>
         </is>
       </c>
-      <c r="F18" s="45" t="inlineStr">
+      <c r="F17" s="53" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G18" s="45" t="inlineStr">
+      <c r="G17" s="53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H18" s="45" t="inlineStr">
+      <c r="H17" s="53" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I18" s="45" t="inlineStr">
+      <c r="I17" s="53" t="inlineStr">
         <is>
           <t>Results→recommendation connector.</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="B19" s="46" t="inlineStr">
+      <c r="J17" s="49" t="n"/>
+      <c r="K17" s="49" t="n"/>
+      <c r="L17" s="49" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="49" t="n"/>
+      <c r="B18" s="54" t="inlineStr">
         <is>
           <t>Acs3</t>
         </is>
       </c>
-      <c r="C19" s="46" t="inlineStr">
+      <c r="C18" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D19" s="46" t="inlineStr">
+      <c r="D18" s="54" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="E19" s="46" t="inlineStr">
+      <c r="E18" s="54" t="inlineStr">
         <is>
           <t>In conclusion, the number of rooted...</t>
         </is>
       </c>
-      <c r="F19" s="46" t="inlineStr">
+      <c r="F18" s="54" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G19" s="46" t="inlineStr">
+      <c r="G18" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H19" s="46" t="inlineStr">
+      <c r="H18" s="54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I19" s="46" t="inlineStr">
+      <c r="I18" s="54" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="B20" s="45" t="inlineStr">
+      <c r="J18" s="49" t="n"/>
+      <c r="K18" s="49" t="n"/>
+      <c r="L18" s="49" t="n"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="49" t="n"/>
+      <c r="B19" s="53" t="inlineStr">
         <is>
           <t>Acs7</t>
         </is>
       </c>
-      <c r="C20" s="45" t="inlineStr">
+      <c r="C19" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D20" s="45" t="inlineStr">
+      <c r="D19" s="53" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="E20" s="45" t="inlineStr">
+      <c r="E19" s="53" t="inlineStr">
         <is>
           <t>In conclusion, the use of rice hull...</t>
         </is>
       </c>
-      <c r="F20" s="45" t="inlineStr">
+      <c r="F19" s="53" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G20" s="45" t="inlineStr">
+      <c r="G19" s="53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H20" s="45" t="inlineStr">
+      <c r="H19" s="53" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I20" s="45" t="inlineStr">
+      <c r="I19" s="53" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="B21" s="46" t="inlineStr">
+      <c r="J19" s="49" t="n"/>
+      <c r="K19" s="49" t="n"/>
+      <c r="L19" s="49" t="n"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="49" t="n"/>
+      <c r="B20" s="54" t="inlineStr">
         <is>
           <t>Acs10</t>
         </is>
       </c>
-      <c r="C21" s="46" t="inlineStr">
+      <c r="C20" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D21" s="46" t="inlineStr">
+      <c r="D20" s="54" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="E21" s="46" t="inlineStr">
+      <c r="E20" s="54" t="inlineStr">
         <is>
           <t>In conclusion, T3:...</t>
         </is>
       </c>
-      <c r="F21" s="46" t="inlineStr">
+      <c r="F20" s="54" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G21" s="46" t="inlineStr">
+      <c r="G20" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H21" s="46" t="inlineStr">
+      <c r="H20" s="54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I21" s="46" t="inlineStr">
+      <c r="I20" s="54" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="B22" s="45" t="inlineStr">
+      <c r="J20" s="49" t="n"/>
+      <c r="K20" s="49" t="n"/>
+      <c r="L20" s="49" t="n"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="49" t="n"/>
+      <c r="B21" s="53" t="inlineStr">
         <is>
           <t>Aas3</t>
         </is>
       </c>
-      <c r="C22" s="45" t="inlineStr">
+      <c r="C21" s="53" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D22" s="45" t="inlineStr">
+      <c r="D21" s="53" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="E22" s="45" t="inlineStr">
+      <c r="E21" s="53" t="inlineStr">
         <is>
           <t>In conclusion, proved the treatment 1...</t>
         </is>
       </c>
-      <c r="F22" s="45" t="inlineStr">
+      <c r="F21" s="53" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G22" s="45" t="inlineStr">
+      <c r="G21" s="53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H22" s="45" t="inlineStr">
+      <c r="H21" s="53" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I22" s="45" t="inlineStr">
+      <c r="I21" s="53" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="B23" s="46" t="inlineStr">
+      <c r="J21" s="49" t="n"/>
+      <c r="K21" s="49" t="n"/>
+      <c r="L21" s="49" t="n"/>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="49" t="n"/>
+      <c r="B22" s="54" t="inlineStr">
         <is>
           <t>Aas10</t>
         </is>
       </c>
-      <c r="C23" s="46" t="inlineStr">
+      <c r="C22" s="54" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D23" s="46" t="inlineStr">
+      <c r="D22" s="54" t="inlineStr">
         <is>
           <t>In conclusion</t>
         </is>
       </c>
-      <c r="E23" s="46" t="inlineStr">
+      <c r="E22" s="54" t="inlineStr">
         <is>
           <t>In conclusion, based on the results, it can be stated...</t>
         </is>
       </c>
-      <c r="F23" s="46" t="inlineStr">
+      <c r="F22" s="54" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="G23" s="46" t="inlineStr">
+      <c r="G22" s="54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H23" s="46" t="inlineStr">
+      <c r="H22" s="54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I23" s="46" t="inlineStr">
+      <c r="I22" s="54" t="inlineStr">
         <is>
           <t>Meta-textual framing of conclusion move.</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="40" customHeight="1">
-      <c r="B24" s="47" t="inlineStr">
+      <c r="J22" s="49" t="n"/>
+      <c r="K22" s="49" t="n"/>
+      <c r="L22" s="49" t="n"/>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="49" t="n"/>
+      <c r="B23" s="55" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C24" s="47" t="inlineStr">
+      <c r="C23" s="55" t="inlineStr">
         <is>
           <t>All disciplines</t>
         </is>
       </c>
-      <c r="D24" s="47" t="inlineStr">
+      <c r="D23" s="55" t="inlineStr">
         <is>
           <t>(none)</t>
         </is>
       </c>
-      <c r="E24" s="47" t="inlineStr">
+      <c r="E23" s="55" t="inlineStr">
         <is>
           <t>No "as X suggested", "in our view", "please", "kindly", "with due respect", "one might argue"</t>
         </is>
       </c>
-      <c r="F24" s="47" t="inlineStr">
+      <c r="F23" s="55" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="G24" s="47" t="inlineStr">
+      <c r="G23" s="55" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H24" s="47" t="inlineStr">
+      <c r="H23" s="55" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I24" s="47" t="inlineStr">
+      <c r="I23" s="55" t="inlineStr">
         <is>
           <t>No politeness/deference devices in the 60 abstracts.</t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="40" customHeight="1">
-      <c r="B25" s="47" t="inlineStr">
+      <c r="J23" s="49" t="n"/>
+      <c r="K23" s="49" t="n"/>
+      <c r="L23" s="49" t="n"/>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="49" t="n"/>
+      <c r="B24" s="55" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="C25" s="47" t="inlineStr">
+      <c r="C24" s="55" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D25" s="47" t="inlineStr">
+      <c r="D24" s="55" t="inlineStr">
         <is>
           <t>regarding / with regard to / overall / first-second</t>
         </is>
       </c>
-      <c r="E25" s="47" t="inlineStr">
+      <c r="E24" s="55" t="inlineStr">
         <is>
           <t>Common in VM KAP and ranking sentences</t>
         </is>
       </c>
-      <c r="F25" s="47" t="inlineStr">
+      <c r="F24" s="55" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G25" s="47" t="inlineStr">
+      <c r="G24" s="55" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H25" s="47" t="inlineStr">
+      <c r="H24" s="55" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I25" s="47" t="inlineStr">
+      <c r="I24" s="55" t="inlineStr">
         <is>
           <t>Topic prepositions and ordinal ranking of results are NOT discourse-organization function. Left untagged.</t>
         </is>
       </c>
+      <c r="J24" s="49" t="n"/>
+      <c r="K24" s="49" t="n"/>
+      <c r="L24" s="49" t="n"/>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="49" t="n"/>
+      <c r="B25" s="55" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="C25" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D25" s="55" t="inlineStr">
+        <is>
+          <t>should / recommended (FP-Rec)</t>
+        </is>
+      </c>
+      <c r="E25" s="55" t="inlineStr">
+        <is>
+          <t>See Rejected Candidates</t>
+        </is>
+      </c>
+      <c r="F25" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H25" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="55" t="inlineStr">
+        <is>
+          <t>Deontic prescriptions. Reject reason FP-Rec, not Layer 2 P or DO.</t>
+        </is>
+      </c>
+      <c r="J25" s="49" t="n"/>
+      <c r="K25" s="49" t="n"/>
+      <c r="L25" s="49" t="n"/>
     </row>
     <row r="26" ht="40" customHeight="1">
-      <c r="B26" s="47" t="inlineStr">
-        <is>
-          <t>NOTE</t>
-        </is>
-      </c>
-      <c r="C26" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D26" s="47" t="inlineStr">
-        <is>
-          <t>should / recommended (FP-Rec)</t>
-        </is>
-      </c>
-      <c r="E26" s="47" t="inlineStr">
-        <is>
-          <t>See Rejected Candidates</t>
-        </is>
-      </c>
-      <c r="F26" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="47" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H26" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="47" t="inlineStr">
-        <is>
-          <t>Deontic prescriptions. Reject reason FP-Rec, not Layer 2 P or DO.</t>
-        </is>
-      </c>
+      <c r="A26" s="49" t="n"/>
+      <c r="B26" s="49" t="n"/>
+      <c r="C26" s="49" t="n"/>
+      <c r="D26" s="49" t="n"/>
+      <c r="E26" s="49" t="n"/>
+      <c r="F26" s="49" t="n"/>
+      <c r="G26" s="49" t="n"/>
+      <c r="H26" s="49" t="n"/>
+      <c r="I26" s="49" t="n"/>
+      <c r="J26" s="49" t="n"/>
+      <c r="K26" s="49" t="n"/>
+      <c r="L26" s="49" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="49" t="n"/>
+      <c r="B27" s="49" t="n"/>
+      <c r="C27" s="49" t="n"/>
+      <c r="D27" s="49" t="n"/>
+      <c r="E27" s="49" t="n"/>
+      <c r="F27" s="49" t="n"/>
+      <c r="G27" s="49" t="n"/>
+      <c r="H27" s="49" t="n"/>
+      <c r="I27" s="49" t="n"/>
+      <c r="J27" s="49" t="n"/>
+      <c r="K27" s="49" t="n"/>
+      <c r="L27" s="49" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="n"/>
+      <c r="B28" s="49" t="n"/>
+      <c r="C28" s="49" t="n"/>
+      <c r="D28" s="49" t="n"/>
+      <c r="E28" s="49" t="n"/>
+      <c r="F28" s="49" t="n"/>
+      <c r="G28" s="49" t="n"/>
+      <c r="H28" s="49" t="n"/>
+      <c r="I28" s="49" t="n"/>
+      <c r="J28" s="49" t="n"/>
+      <c r="K28" s="49" t="n"/>
+      <c r="L28" s="49" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="n"/>
+      <c r="B29" s="49" t="n"/>
+      <c r="C29" s="49" t="n"/>
+      <c r="D29" s="49" t="n"/>
+      <c r="E29" s="49" t="n"/>
+      <c r="F29" s="49" t="n"/>
+      <c r="G29" s="49" t="n"/>
+      <c r="H29" s="49" t="n"/>
+      <c r="I29" s="49" t="n"/>
+      <c r="J29" s="49" t="n"/>
+      <c r="K29" s="49" t="n"/>
+      <c r="L29" s="49" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="n"/>
+      <c r="B30" s="49" t="n"/>
+      <c r="C30" s="49" t="n"/>
+      <c r="D30" s="49" t="n"/>
+      <c r="E30" s="49" t="n"/>
+      <c r="F30" s="49" t="n"/>
+      <c r="G30" s="49" t="n"/>
+      <c r="H30" s="49" t="n"/>
+      <c r="I30" s="49" t="n"/>
+      <c r="J30" s="49" t="n"/>
+      <c r="K30" s="49" t="n"/>
+      <c r="L30" s="49" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Excel: apply full Hedges design to rows 65-69
Rows 65-69 were missing row height (45), zebra fill, token highlight
(red for Lexical), function color, borders, clause/notes fonts, and
alignment. Matched existing sheet pattern. No other sheets had the
same incomplete-row miss.
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -5442,216 +5442,216 @@
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="B65" t="inlineStr">
+    <row r="65" ht="45" customHeight="1">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>B11</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D65" t="n">
+      <c r="D65" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="18" t="inlineStr">
         <is>
           <t>Hence, this study aimed to investigate the presence of potential mycobacterial infections in cultivated milkfish collected from fish-supplying areas of Pampanga.</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="19" t="inlineStr">
         <is>
           <t>potential</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G65" s="5" t="inlineStr">
         <is>
           <t>Lexical Hedges</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H65" s="20" t="inlineStr">
         <is>
           <t>EC</t>
         </is>
       </c>
-      <c r="I65" t="n">
+      <c r="I65" s="5" t="n">
         <v>256</v>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="J65" s="21" t="inlineStr">
         <is>
           <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'presence of mycobacterial infections' asserts existence; 'potential mycobacterial infections' marks them as possible.</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="B66" t="inlineStr">
+    <row r="66" ht="45" customHeight="1">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>B12</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="6" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D66" t="n">
+      <c r="D66" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E66" s="22" t="inlineStr">
         <is>
           <t>Hence, lactic acid bacteria (LAB) have emerged as a focal point due to their potential quorum quenching (QQ) activities.</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="19" t="inlineStr">
         <is>
           <t>potential</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G66" s="6" t="inlineStr">
         <is>
           <t>Lexical Hedges</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H66" s="20" t="inlineStr">
         <is>
           <t>EC</t>
         </is>
       </c>
-      <c r="I66" t="n">
+      <c r="I66" s="6" t="n">
         <v>149</v>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="J66" s="23" t="inlineStr">
         <is>
           <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'their quorum quenching activities' asserts the activities exist.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="B67" t="inlineStr">
+    <row r="67" ht="45" customHeight="1">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>B16</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="D67" t="n">
+      <c r="D67" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E67" t="inlineStr">
+      <c r="E67" s="18" t="inlineStr">
         <is>
           <t>The increasing popularity of SHC or “ukay-ukay” in the Philippines, coupled with potential public health concerns associated with transmitting pathogenic bacteria, emphasized this research’s need.</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="19" t="inlineStr">
         <is>
           <t>potential</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G67" s="5" t="inlineStr">
         <is>
           <t>Lexical Hedges</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H67" s="20" t="inlineStr">
         <is>
           <t>EC</t>
         </is>
       </c>
-      <c r="I67" t="n">
+      <c r="I67" s="5" t="n">
         <v>223</v>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="J67" s="21" t="inlineStr">
         <is>
           <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'public health concerns' asserted as fact vs possible. Same abstract also codes conclusion-position 'potential public health risks' as EC.</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="B68" t="inlineStr">
+    <row r="68" ht="45" customHeight="1">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>VM9</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>Veterinary Medicine</t>
         </is>
       </c>
-      <c r="D68" t="n">
+      <c r="D68" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E68" s="22" t="inlineStr">
         <is>
           <t>Its persistence in marine environments, particularly in the form of microplastics, posed potential health risks to aquatic species and humans through seafood consumption.</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F68" s="19" t="inlineStr">
         <is>
           <t>potential</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>Lexical Hedges</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="H68" s="20" t="inlineStr">
         <is>
           <t>EC</t>
         </is>
       </c>
-      <c r="I68" t="n">
+      <c r="I68" s="6" t="n">
         <v>430</v>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="J68" s="23" t="inlineStr">
         <is>
           <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'posed health risks' asserts risks as fact.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" t="inlineStr">
+    <row r="69" ht="45" customHeight="1">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>Aas5</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D69" t="n">
+      <c r="D69" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E69" s="18" t="inlineStr">
         <is>
           <t>Fortunately, insect farming can be seen as a potential solution for filling the protein gap for feed and food resources in a more sustainable manned compared to other animal protein sources.</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="19" t="inlineStr">
         <is>
           <t>potential</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G69" s="5" t="inlineStr">
         <is>
           <t>Lexical Hedges</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H69" s="20" t="inlineStr">
         <is>
           <t>EC</t>
         </is>
       </c>
-      <c r="I69" t="n">
+      <c r="I69" s="5" t="n">
         <v>316</v>
       </c>
-      <c r="J69" t="inlineStr">
+      <c r="J69" s="21" t="inlineStr">
         <is>
           <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'a solution' is stronger endorsement than 'a potential solution'. Multi-hedge isolation: 'can' already coded EC in same sentence; 'potential' independently softens.</t>
         </is>

</xml_diff>

<commit_message>
Excel: add Table 7 outcome cross-tab and definitions
On Summary and Outcome Type sheets. Counts match thesis (60 abstracts).
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -137,8 +137,27 @@
       <color rgb="008C8A84"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -213,8 +232,13 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -267,11 +291,19 @@
       </bottom>
     </border>
     <border/>
+    <border>
+      <top style="medium"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="medium"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -388,6 +420,27 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -754,19 +807,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H101"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="88" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -781,6 +835,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -925,6 +980,8 @@
         <v>0.47</v>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -1018,6 +1075,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -1117,6 +1176,8 @@
         <v>33</v>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -1186,6 +1247,8 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="16" t="inlineStr">
         <is>
@@ -1193,6 +1256,8 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -2789,6 +2854,267 @@
       <c r="G101" s="5" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="63" t="inlineStr">
+        <is>
+          <t>Outcome Type by Discipline (Table 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="64" t="inlineStr">
+        <is>
+          <t>Counts are abstracts (one outcome type per abstract). Matches thesis Table 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="65" t="inlineStr">
+        <is>
+          <t>Outcome Type</t>
+        </is>
+      </c>
+      <c r="C107" s="65" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D107" s="65" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="E107" s="65" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="F107" s="65" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="66" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="C108" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" s="67" t="n">
+        <v>8</v>
+      </c>
+      <c r="E108" s="67" t="n">
+        <v>7</v>
+      </c>
+      <c r="F108" s="67" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="68" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="C109" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="D109" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="E109" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="F109" s="69" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C110" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D110" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E110" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="F110" s="67" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="68" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="C111" s="69" t="n">
+        <v>14</v>
+      </c>
+      <c r="D111" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E111" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="F111" s="69" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="66" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C112" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E112" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F112" s="67" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="70" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C113" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="D113" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="E113" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="F113" s="71" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="63" t="inlineStr">
+        <is>
+          <t>Outcome Type Definitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="64" t="inlineStr">
+        <is>
+          <t>Same definitions used in thesis Part IV. Not hedge types.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="65" t="inlineStr">
+        <is>
+          <t>Outcome Type</t>
+        </is>
+      </c>
+      <c r="C119" s="65" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="D119" s="65" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="45" customHeight="1">
+      <c r="B120" s="66" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="C120" s="67" t="n">
+        <v>15</v>
+      </c>
+      <c r="D120" s="66" t="inlineStr">
+        <is>
+          <t>Presence or absence findings or clear yes/no outcomes (e.g., zone of inhibition vs none, pathogen detected vs not, positive vs negative diagnostic result).</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="45" customHeight="1">
+      <c r="B121" s="68" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="C121" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="D121" s="68" t="inlineStr">
+        <is>
+          <t>Graded quantities such as means, yields, rates, concentrations, or growth measures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="45" customHeight="1">
+      <c r="B122" s="66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C122" s="67" t="n">
+        <v>9</v>
+      </c>
+      <c r="D122" s="66" t="inlineStr">
+        <is>
+          <t>Abstract combines more than one outcome style (e.g., binary plus continuous, or continuous plus a null test).</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="45" customHeight="1">
+      <c r="B123" s="68" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="C123" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="D123" s="68" t="inlineStr">
+        <is>
+          <t>Abstract explicitly reports non-significance, no significant difference, or a null statistical result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="45" customHeight="1">
+      <c r="B124" s="66" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C124" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="D124" s="66" t="inlineStr">
+        <is>
+          <t>Results language does not fit the four boxes cleanly (e.g., descriptive profiles, rankings, or designs that are not clearly binary, continuous, mixed, or null).</t>
         </is>
       </c>
     </row>
@@ -9165,15 +9491,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="88" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11129,6 +11455,267 @@
       <c r="J67" s="49" t="n"/>
       <c r="K67" s="49" t="n"/>
       <c r="L67" s="49" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="63" t="inlineStr">
+        <is>
+          <t>Outcome Type by Discipline (Table 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="64" t="inlineStr">
+        <is>
+          <t>Counts are abstracts. One outcome type per abstract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="65" t="inlineStr">
+        <is>
+          <t>Outcome Type</t>
+        </is>
+      </c>
+      <c r="C73" s="65" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D73" s="65" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="E73" s="65" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="F73" s="65" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="66" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="C74" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="67" t="n">
+        <v>8</v>
+      </c>
+      <c r="E74" s="67" t="n">
+        <v>7</v>
+      </c>
+      <c r="F74" s="67" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="68" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="C75" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="D75" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="E75" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" s="69" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C76" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D76" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E76" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="F76" s="67" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="68" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="C77" s="69" t="n">
+        <v>14</v>
+      </c>
+      <c r="D77" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="F77" s="69" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="66" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C78" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E78" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" s="67" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="70" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C79" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="D79" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="E79" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="F79" s="71" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="63" t="inlineStr">
+        <is>
+          <t>Outcome Type Definitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="64" t="inlineStr">
+        <is>
+          <t>Same definitions used in thesis Part IV. These are not hedge types.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="65" t="inlineStr">
+        <is>
+          <t>Outcome Type</t>
+        </is>
+      </c>
+      <c r="C85" s="65" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="D85" s="65" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="45" customHeight="1">
+      <c r="B86" s="66" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="C86" s="67" t="n">
+        <v>15</v>
+      </c>
+      <c r="D86" s="66" t="inlineStr">
+        <is>
+          <t>Presence or absence findings or clear yes/no outcomes (e.g., zone of inhibition vs none, pathogen detected vs not, positive vs negative diagnostic result).</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="45" customHeight="1">
+      <c r="B87" s="68" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="C87" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="D87" s="68" t="inlineStr">
+        <is>
+          <t>Graded quantities such as means, yields, rates, concentrations, or growth measures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="45" customHeight="1">
+      <c r="B88" s="66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C88" s="67" t="n">
+        <v>9</v>
+      </c>
+      <c r="D88" s="66" t="inlineStr">
+        <is>
+          <t>Abstract combines more than one outcome style (e.g., binary plus continuous, or continuous plus a null test).</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="45" customHeight="1">
+      <c r="B89" s="68" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="C89" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="D89" s="68" t="inlineStr">
+        <is>
+          <t>Abstract explicitly reports non-significance, no significant difference, or a null statistical result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="45" customHeight="1">
+      <c r="B90" s="66" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C90" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="D90" s="66" t="inlineStr">
+        <is>
+          <t>Results language does not fit the four boxes cleanly (e.g., descriptive profiles, rankings, or designs that are not clearly binary, continuous, mixed, or null).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Excel: keep Table 7 and definitions on Summary only
Removed the duplicate block from the Outcome Type sheet.
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H124"/>
+  <dimension ref="B2:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,6 @@
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -835,7 +834,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -980,8 +978,6 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -1075,8 +1071,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -1176,8 +1170,6 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -1247,8 +1239,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36"/>
     <row r="37">
       <c r="B37" s="16" t="inlineStr">
         <is>
@@ -1256,8 +1246,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40">
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -9491,7 +9479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -11456,267 +11444,13 @@
       <c r="K67" s="49" t="n"/>
       <c r="L67" s="49" t="n"/>
     </row>
-    <row r="70">
-      <c r="B70" s="63" t="inlineStr">
-        <is>
-          <t>Outcome Type by Discipline (Table 7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="64" t="inlineStr">
-        <is>
-          <t>Counts are abstracts. One outcome type per abstract.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" s="65" t="inlineStr">
-        <is>
-          <t>Outcome Type</t>
-        </is>
-      </c>
-      <c r="C73" s="65" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="D73" s="65" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="E73" s="65" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="F73" s="65" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="66" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="C74" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="D74" s="67" t="n">
-        <v>8</v>
-      </c>
-      <c r="E74" s="67" t="n">
-        <v>7</v>
-      </c>
-      <c r="F74" s="67" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" s="68" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="C75" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="D75" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="E75" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="F75" s="69" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="66" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="C76" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="D76" s="67" t="n">
-        <v>3</v>
-      </c>
-      <c r="E76" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="F76" s="67" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="B77" s="68" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="C77" s="69" t="n">
-        <v>14</v>
-      </c>
-      <c r="D77" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="E77" s="69" t="n">
-        <v>5</v>
-      </c>
-      <c r="F77" s="69" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="66" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C78" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="D78" s="67" t="n">
-        <v>3</v>
-      </c>
-      <c r="E78" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="F78" s="67" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" s="70" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C79" s="71" t="n">
-        <v>20</v>
-      </c>
-      <c r="D79" s="71" t="n">
-        <v>20</v>
-      </c>
-      <c r="E79" s="71" t="n">
-        <v>20</v>
-      </c>
-      <c r="F79" s="71" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="B82" s="63" t="inlineStr">
-        <is>
-          <t>Outcome Type Definitions</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="B83" s="64" t="inlineStr">
-        <is>
-          <t>Same definitions used in thesis Part IV. These are not hedge types.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="B85" s="65" t="inlineStr">
-        <is>
-          <t>Outcome Type</t>
-        </is>
-      </c>
-      <c r="C85" s="65" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="D85" s="65" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="45" customHeight="1">
-      <c r="B86" s="66" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="C86" s="67" t="n">
-        <v>15</v>
-      </c>
-      <c r="D86" s="66" t="inlineStr">
-        <is>
-          <t>Presence or absence findings or clear yes/no outcomes (e.g., zone of inhibition vs none, pathogen detected vs not, positive vs negative diagnostic result).</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="45" customHeight="1">
-      <c r="B87" s="68" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="C87" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="D87" s="68" t="inlineStr">
-        <is>
-          <t>Graded quantities such as means, yields, rates, concentrations, or growth measures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="45" customHeight="1">
-      <c r="B88" s="66" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="C88" s="67" t="n">
-        <v>9</v>
-      </c>
-      <c r="D88" s="66" t="inlineStr">
-        <is>
-          <t>Abstract combines more than one outcome style (e.g., binary plus continuous, or continuous plus a null test).</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="45" customHeight="1">
-      <c r="B89" s="68" t="inlineStr">
-        <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="C89" s="69" t="n">
-        <v>21</v>
-      </c>
-      <c r="D89" s="68" t="inlineStr">
-        <is>
-          <t>Abstract explicitly reports non-significance, no significant difference, or a null statistical result.</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="45" customHeight="1">
-      <c r="B90" s="66" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C90" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="D90" s="66" t="inlineStr">
-        <is>
-          <t>Results language does not fit the four boxes cleanly (e.g., descriptive profiles, rankings, or designs that are not clearly binary, continuous, mixed, or null).</t>
-        </is>
-      </c>
-    </row>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="86" ht="45" customHeight="1"/>
+    <row r="87" ht="45" customHeight="1"/>
+    <row r="88" ht="45" customHeight="1"/>
+    <row r="89" ht="45" customHeight="1"/>
+    <row r="90" ht="45" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel Summary: add Table 3 hedge token inventory by form
15 surface forms with type, count, and share of 65. Matches thesis.
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -807,19 +807,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H124"/>
+  <dimension ref="A1:H146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="88" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -834,6 +835,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -978,6 +980,8 @@
         <v>0.47</v>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -1071,6 +1075,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -1170,6 +1176,8 @@
         <v>33</v>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -1239,6 +1247,8 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="16" t="inlineStr">
         <is>
@@ -1246,6 +1256,8 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -2845,262 +2857,621 @@
         </is>
       </c>
     </row>
+    <row r="102"/>
+    <row r="103"/>
     <row r="104">
       <c r="B104" s="63" t="inlineStr">
         <is>
-          <t>Outcome Type by Discipline (Table 7)</t>
+          <t>Hedge Token Inventory by Form (Table 3)</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" s="64" t="inlineStr">
         <is>
-          <t>Counts are abstracts (one outcome type per abstract). Matches thesis Table 7.</t>
+          <t>Every retained surface form with Layer 1 type and count. Sums to 65. Matches thesis Table 3.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="65" t="inlineStr">
         <is>
-          <t>Outcome Type</t>
+          <t>Hedge form</t>
         </is>
       </c>
       <c r="C107" s="65" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Layer 1 type</t>
         </is>
       </c>
       <c r="D107" s="65" t="inlineStr">
         <is>
-          <t>Veterinary Medicine</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="E107" s="65" t="inlineStr">
         <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="F107" s="65" t="inlineStr">
-        <is>
-          <t>Total</t>
+          <t>% of total hedges</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" s="66" t="inlineStr">
         <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="C108" s="67" t="n">
-        <v>0</v>
+          <t>potential</t>
+        </is>
+      </c>
+      <c r="C108" s="66" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
       </c>
       <c r="D108" s="67" t="n">
-        <v>8</v>
-      </c>
-      <c r="E108" s="67" t="n">
-        <v>7</v>
-      </c>
-      <c r="F108" s="67" t="n">
-        <v>15</v>
+        <v>19</v>
+      </c>
+      <c r="E108" s="67" t="inlineStr">
+        <is>
+          <t>29.2%</t>
+        </is>
       </c>
     </row>
     <row r="109">
       <c r="B109" s="68" t="inlineStr">
         <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="C109" s="69" t="n">
-        <v>4</v>
+          <t>suggests</t>
+        </is>
+      </c>
+      <c r="C109" s="68" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
       </c>
       <c r="D109" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="E109" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="F109" s="69" t="n">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="E109" s="69" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" s="66" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="C110" s="67" t="n">
-        <v>2</v>
+          <t>suggest</t>
+        </is>
+      </c>
+      <c r="C110" s="66" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
       </c>
       <c r="D110" s="67" t="n">
         <v>3</v>
       </c>
-      <c r="E110" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="F110" s="67" t="n">
-        <v>9</v>
+      <c r="E110" s="67" t="inlineStr">
+        <is>
+          <t>4.6%</t>
+        </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" s="68" t="inlineStr">
         <is>
-          <t>Null/NS</t>
-        </is>
-      </c>
-      <c r="C111" s="69" t="n">
-        <v>14</v>
+          <t>suggesting</t>
+        </is>
+      </c>
+      <c r="C111" s="68" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
       </c>
       <c r="D111" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="E111" s="69" t="n">
-        <v>5</v>
-      </c>
-      <c r="F111" s="69" t="n">
-        <v>21</v>
+        <v>3</v>
+      </c>
+      <c r="E111" s="69" t="inlineStr">
+        <is>
+          <t>4.6%</t>
+        </is>
       </c>
     </row>
     <row r="112">
       <c r="B112" s="66" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C112" s="67" t="n">
-        <v>0</v>
+          <t>implies</t>
+        </is>
+      </c>
+      <c r="C112" s="66" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
       </c>
       <c r="D112" s="67" t="n">
-        <v>3</v>
-      </c>
-      <c r="E112" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="F112" s="67" t="n">
-        <v>5</v>
+      <c r="E112" s="67" t="inlineStr">
+        <is>
+          <t>3.1%</t>
+        </is>
       </c>
     </row>
     <row r="113">
-      <c r="B113" s="70" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C113" s="71" t="n">
-        <v>20</v>
-      </c>
-      <c r="D113" s="71" t="n">
-        <v>20</v>
-      </c>
-      <c r="E113" s="71" t="n">
-        <v>20</v>
-      </c>
-      <c r="F113" s="71" t="n">
-        <v>60</v>
+      <c r="B113" s="68" t="inlineStr">
+        <is>
+          <t>indicating</t>
+        </is>
+      </c>
+      <c r="C113" s="68" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
+      </c>
+      <c r="D113" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E113" s="69" t="inlineStr">
+        <is>
+          <t>3.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="66" t="inlineStr">
+        <is>
+          <t>likely</t>
+        </is>
+      </c>
+      <c r="C114" s="66" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
+      </c>
+      <c r="D114" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E114" s="67" t="inlineStr">
+        <is>
+          <t>3.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="68" t="inlineStr">
+        <is>
+          <t>implying</t>
+        </is>
+      </c>
+      <c r="C115" s="68" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
+      </c>
+      <c r="D115" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="E115" s="69" t="inlineStr">
+        <is>
+          <t>1.5%</t>
+        </is>
       </c>
     </row>
     <row r="116">
-      <c r="B116" s="63" t="inlineStr">
-        <is>
-          <t>Outcome Type Definitions</t>
+      <c r="B116" s="66" t="inlineStr">
+        <is>
+          <t>inferring</t>
+        </is>
+      </c>
+      <c r="C116" s="66" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
+      </c>
+      <c r="D116" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" s="67" t="inlineStr">
+        <is>
+          <t>1.5%</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="B117" s="64" t="inlineStr">
-        <is>
-          <t>Same definitions used in thesis Part IV. Not hedge types.</t>
+      <c r="B117" s="68" t="inlineStr">
+        <is>
+          <t>possible</t>
+        </is>
+      </c>
+      <c r="C117" s="68" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
+      </c>
+      <c r="D117" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="E117" s="69" t="inlineStr">
+        <is>
+          <t>1.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="66" t="inlineStr">
+        <is>
+          <t>can</t>
+        </is>
+      </c>
+      <c r="C118" s="66" t="inlineStr">
+        <is>
+          <t>Modal Verbs</t>
+        </is>
+      </c>
+      <c r="D118" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="E118" s="67" t="inlineStr">
+        <is>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="B119" s="65" t="inlineStr">
-        <is>
-          <t>Outcome Type</t>
-        </is>
-      </c>
-      <c r="C119" s="65" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="D119" s="65" t="inlineStr">
-        <is>
-          <t>Meaning</t>
+      <c r="B119" s="68" t="inlineStr">
+        <is>
+          <t>could</t>
+        </is>
+      </c>
+      <c r="C119" s="68" t="inlineStr">
+        <is>
+          <t>Modal Verbs</t>
+        </is>
+      </c>
+      <c r="D119" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="E119" s="69" t="inlineStr">
+        <is>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="120" ht="45" customHeight="1">
       <c r="B120" s="66" t="inlineStr">
         <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="C120" s="67" t="n">
-        <v>15</v>
-      </c>
-      <c r="D120" s="66" t="inlineStr">
-        <is>
-          <t>Presence or absence findings or clear yes/no outcomes (e.g., zone of inhibition vs none, pathogen detected vs not, positive vs negative diagnostic result).</t>
+          <t>may</t>
+        </is>
+      </c>
+      <c r="C120" s="66" t="inlineStr">
+        <is>
+          <t>Modal Verbs</t>
+        </is>
+      </c>
+      <c r="D120" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="E120" s="67" t="inlineStr">
+        <is>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="121" ht="45" customHeight="1">
       <c r="B121" s="68" t="inlineStr">
         <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="C121" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="D121" s="68" t="inlineStr">
-        <is>
-          <t>Graded quantities such as means, yields, rates, concentrations, or growth measures.</t>
+          <t>might</t>
+        </is>
+      </c>
+      <c r="C121" s="68" t="inlineStr">
+        <is>
+          <t>Modal Verbs</t>
+        </is>
+      </c>
+      <c r="D121" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="E121" s="69" t="inlineStr">
+        <is>
+          <t>4.6%</t>
         </is>
       </c>
     </row>
     <row r="122" ht="45" customHeight="1">
       <c r="B122" s="66" t="inlineStr">
         <is>
+          <t>potentially</t>
+        </is>
+      </c>
+      <c r="C122" s="66" t="inlineStr">
+        <is>
+          <t>Adverbial Hedges</t>
+        </is>
+      </c>
+      <c r="D122" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E122" s="67" t="inlineStr">
+        <is>
+          <t>4.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="45" customHeight="1">
+      <c r="B123" s="70" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C123" s="70" t="inlineStr"/>
+      <c r="D123" s="71" t="n">
+        <v>65</v>
+      </c>
+      <c r="E123" s="71" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="45" customHeight="1"/>
+    <row r="126">
+      <c r="B126" s="63" t="inlineStr">
+        <is>
+          <t>Outcome Type by Discipline (Table 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" s="64" t="inlineStr">
+        <is>
+          <t>Counts are abstracts (one outcome type per abstract). Matches thesis Table 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128"/>
+    <row r="129">
+      <c r="B129" s="65" t="inlineStr">
+        <is>
+          <t>Outcome Type</t>
+        </is>
+      </c>
+      <c r="C129" s="65" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D129" s="65" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="E129" s="65" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="F129" s="65" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" s="66" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="C130" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D130" s="67" t="n">
+        <v>8</v>
+      </c>
+      <c r="E130" s="67" t="n">
+        <v>7</v>
+      </c>
+      <c r="F130" s="67" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="B131" s="68" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="C131" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="D131" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="E131" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="F131" s="69" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" s="66" t="inlineStr">
+        <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="C122" s="67" t="n">
+      <c r="C132" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D132" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E132" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="F132" s="67" t="n">
         <v>9</v>
       </c>
-      <c r="D122" s="66" t="inlineStr">
+    </row>
+    <row r="133">
+      <c r="B133" s="68" t="inlineStr">
+        <is>
+          <t>Null/NS</t>
+        </is>
+      </c>
+      <c r="C133" s="69" t="n">
+        <v>14</v>
+      </c>
+      <c r="D133" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E133" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="F133" s="69" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="B134" s="66" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C134" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E134" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F134" s="67" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="B135" s="70" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C135" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="D135" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="E135" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="F135" s="71" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138">
+      <c r="B138" s="63" t="inlineStr">
+        <is>
+          <t>Outcome Type Definitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="B139" s="64" t="inlineStr">
+        <is>
+          <t>Same definitions used in thesis Part IV. Not hedge types.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140"/>
+    <row r="141">
+      <c r="B141" s="65" t="inlineStr">
+        <is>
+          <t>Outcome Type</t>
+        </is>
+      </c>
+      <c r="C141" s="65" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="D141" s="65" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="B142" s="66" t="inlineStr">
+        <is>
+          <t>Binary</t>
+        </is>
+      </c>
+      <c r="C142" s="67" t="n">
+        <v>15</v>
+      </c>
+      <c r="D142" s="66" t="inlineStr">
+        <is>
+          <t>Presence or absence findings or clear yes/no outcomes (e.g., zone of inhibition vs none, pathogen detected vs not, positive vs negative diagnostic result).</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="B143" s="68" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="C143" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="D143" s="68" t="inlineStr">
+        <is>
+          <t>Graded quantities such as means, yields, rates, concentrations, or growth measures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="B144" s="66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C144" s="67" t="n">
+        <v>9</v>
+      </c>
+      <c r="D144" s="66" t="inlineStr">
         <is>
           <t>Abstract combines more than one outcome style (e.g., binary plus continuous, or continuous plus a null test).</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="45" customHeight="1">
-      <c r="B123" s="68" t="inlineStr">
+    <row r="145">
+      <c r="B145" s="68" t="inlineStr">
         <is>
           <t>Null/NS</t>
         </is>
       </c>
-      <c r="C123" s="69" t="n">
+      <c r="C145" s="69" t="n">
         <v>21</v>
       </c>
-      <c r="D123" s="68" t="inlineStr">
+      <c r="D145" s="68" t="inlineStr">
         <is>
           <t>Abstract explicitly reports non-significance, no significant difference, or a null statistical result.</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="45" customHeight="1">
-      <c r="B124" s="66" t="inlineStr">
+    <row r="146">
+      <c r="B146" s="66" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="C124" s="67" t="n">
+      <c r="C146" s="67" t="n">
         <v>5</v>
       </c>
-      <c r="D124" s="66" t="inlineStr">
+      <c r="D146" s="66" t="inlineStr">
         <is>
           <t>Results language does not fit the four boxes cleanly (e.g., descriptive profiles, rankings, or designs that are not clearly binary, continuous, mixed, or null).</t>
         </is>
@@ -9479,7 +9850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -11444,8 +11815,6 @@
       <c r="K67" s="49" t="n"/>
       <c r="L67" s="49" t="n"/>
     </row>
-    <row r="68"/>
-    <row r="69"/>
     <row r="86" ht="45" customHeight="1"/>
     <row r="87" ht="45" customHeight="1"/>
     <row r="88" ht="45" customHeight="1"/>

</xml_diff>

<commit_message>
Draft_050: organic rewrite of patched inserts (no revision narration)
Rewrote decision-rules, reliability, conclusions EC, Scope cross-ref,
Crompton/mitigation, Acs2, and sensitivity closes so they read as
composition rather than later inserts. Appendix A aligned. Excel note
em dashes normalized. Numbers and codes unchanged. Prior drafts retained.
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I136"/>
+  <dimension ref="B2:H136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -829,7 +829,6 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="72" t="inlineStr">
         <is>
@@ -844,7 +843,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="63" t="inlineStr">
         <is>
@@ -989,7 +987,6 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" s="63" t="inlineStr">
         <is>
@@ -1074,7 +1071,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="63" t="inlineStr">
         <is>
@@ -1427,7 +1423,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="B39" s="63" t="inlineStr">
         <is>
@@ -1527,7 +1522,6 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="B47" s="63" t="inlineStr">
         <is>
@@ -1597,7 +1591,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="B53" s="63" t="inlineStr">
         <is>
@@ -1753,7 +1746,6 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="B63" s="63" t="inlineStr">
         <is>
@@ -1860,7 +1852,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="B72" s="64" t="inlineStr">
         <is>
@@ -1868,7 +1859,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
     <row r="74">
       <c r="B74" s="63" t="inlineStr">
         <is>
@@ -3687,7 +3677,7 @@
       </c>
       <c r="J7" s="21" t="inlineStr">
         <is>
-          <t>Lexical hedge: 'indicating unsafe conditions' — inference from coliform presence to a safety judgment, not a restatement of operational meaning. Per indicating rule: inference beyond the data = hedge.</t>
+          <t>Lexical hedge: 'indicating unsafe conditions'  -  inference from coliform presence to a safety judgment, not a restatement of operational meaning. Per indicating rule: inference beyond the data = hedge.</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4150,7 @@
       </c>
       <c r="J18" s="23" t="inlineStr">
         <is>
-          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'presence of mycobacterial infections' asserts existence; 'potential mycobacterial infections' marks them as possible.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment  -  'presence of mycobacterial infections' asserts existence; 'potential mycobacterial infections' marks them as possible.</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4193,7 @@
       </c>
       <c r="J19" s="21" t="inlineStr">
         <is>
-          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'their quorum quenching activities' asserts the activities exist.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment  -  'their quorum quenching activities' asserts the activities exist.</t>
         </is>
       </c>
     </row>
@@ -4418,7 +4408,7 @@
       </c>
       <c r="J24" s="23" t="inlineStr">
         <is>
-          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'public health concerns' asserted as fact vs possible. Same abstract also codes conclusion-position 'potential public health risks' as EC.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment  -  'public health concerns' asserted as fact vs possible. Same abstract also codes conclusion-position 'potential public health risks' as EC.</t>
         </is>
       </c>
     </row>
@@ -5063,7 +5053,7 @@
       </c>
       <c r="J39" s="21" t="inlineStr">
         <is>
-          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'posed health risks' asserts risks as fact.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment  -  'posed health risks' asserts risks as fact.</t>
         </is>
       </c>
     </row>
@@ -5923,7 +5913,7 @@
       </c>
       <c r="J59" s="21" t="inlineStr">
         <is>
-          <t>Modal hedge: 'can effectively promote early growth' — tentative generalization from this study's findings, not an established property. Sits inside a 'suggest' clause softening an overgeneralization.</t>
+          <t>Modal hedge: 'can effectively promote early growth'  -  tentative generalization from this study's findings, not an established property. Sits inside a 'suggest' clause softening an overgeneralization.</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6128,7 @@
       </c>
       <c r="J64" s="23" t="inlineStr">
         <is>
-          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'a solution' is stronger endorsement than 'a potential solution'. Multi-hedge isolation: 'can' already coded EC in same sentence; 'potential' independently softens.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment  -  'a solution' is stronger endorsement than 'a potential solution'. Multi-hedge isolation: 'can' already coded EC in same sentence; 'potential' independently softens.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Draft_053: Stage 1 full corpus pass (no count change), RQ3 restore, knowledge-claim gate
Excel subtitles updated; codebook documents pass outcome.
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -3501,7 +3501,7 @@
     <row r="3">
       <c r="B3" s="48" t="inlineStr">
         <is>
-          <t>Confirmed Layer 1 type + Layer 2 function codes for all retained hedges (n=65 tokens).</t>
+          <t>Confirmed Layer 1 type + Layer 2 function for retained hedges (n=65). Stage 1 retention; Stage 2 function (all EC in this sample).</t>
         </is>
       </c>
     </row>
@@ -6381,7 +6381,7 @@
     <row r="3">
       <c r="B3" s="48" t="inlineStr">
         <is>
-          <t>False-positive hedge candidates rejected under the Working Test, with reason codes.</t>
+          <t>False-positive candidates rejected under Stage 1 exclusions and decision rules (FP-Gen, FP-Rec, FP-Proc, FP-Cap). Full Stage 1 pass: no promotions into retained set.</t>
         </is>
       </c>
     </row>
@@ -11869,7 +11869,7 @@
       <c r="A3" s="49" t="n"/>
       <c r="B3" s="51" t="inlineStr">
         <is>
-          <t>Discourse-organization connectors and politeness scan across 60 abstracts. Hedge? = N for all. Not counted in Layer 1/2 totals.</t>
+          <t>DO connectors and P scan across 60 abstracts. Sequence-only DO and absent P: not retained at Stage 1. Not counted in Layer 1/2 totals.</t>
         </is>
       </c>
       <c r="C3" s="49" t="n"/>
@@ -12976,7 +12976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H44"/>
+  <dimension ref="B1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -12989,6 +12989,7 @@
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="17" t="inlineStr">
         <is>
@@ -12999,7 +13000,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Final coded output for the 60-abstract PSAU corpus, coded per the Hedging Codebook.</t>
+          <t>Final coded output for the 60-abstract PSAU corpus. Stage 1 full pass completed: n=65 retained, all EC at Stage 2; no P forms in corpus; sequence-only DO and FP codes unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Draft_053: replace Layer labels in results tables
Table 3 and Excel Summary use Grammatical type / plain unhedged titles.
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H136"/>
+  <dimension ref="A1:I136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -829,6 +829,7 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="72" t="inlineStr">
         <is>
@@ -843,6 +844,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="63" t="inlineStr">
         <is>
@@ -987,17 +989,18 @@
         <v>0.47</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="B12" s="63" t="inlineStr">
         <is>
-          <t>2. Hedge Type Breakdown (Layer 1) - Table 2</t>
+          <t>2. Hedge Type Breakdown (Type) - Table 2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="65" t="inlineStr">
         <is>
-          <t>Layer 1 Type</t>
+          <t>Grammatical type</t>
         </is>
       </c>
       <c r="C13" s="65" t="inlineStr">
@@ -1071,6 +1074,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="B19" s="63" t="inlineStr">
         <is>
@@ -1093,7 +1097,7 @@
       </c>
       <c r="C21" s="65" t="inlineStr">
         <is>
-          <t>Layer 1 type</t>
+          <t>Grammatical type</t>
         </is>
       </c>
       <c r="D21" s="65" t="inlineStr">
@@ -1423,6 +1427,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="B39" s="63" t="inlineStr">
         <is>
@@ -1522,10 +1527,11 @@
         <v>33</v>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="B47" s="63" t="inlineStr">
         <is>
-          <t>5. Layer 3 - Unhedged Assertion Site Breakdown</t>
+          <t>5. Unhedged Assertion Site Breakdown</t>
         </is>
       </c>
     </row>
@@ -1591,6 +1597,7 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="B53" s="63" t="inlineStr">
         <is>
@@ -1746,6 +1753,7 @@
         <v>60</v>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="B63" s="63" t="inlineStr">
         <is>
@@ -1852,6 +1860,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="B72" s="64" t="inlineStr">
         <is>
@@ -1859,6 +1868,7 @@
         </is>
       </c>
     </row>
+    <row r="73"/>
     <row r="74">
       <c r="B74" s="63" t="inlineStr">
         <is>
@@ -12976,7 +12986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H44"/>
+  <dimension ref="B2:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -12989,7 +12999,6 @@
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Excel: add illustrative Example hedge column for 37 unhedged sites
Draft_056 remains working draft. Appendix C audit clean: 65 EC, 58 FP,
37 UH verb-token greys, no misses or leaks.
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_005.xlsx
+++ b/thesis/007_CompiledResult_Draft_005.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -160,6 +160,20 @@
       <name val="Georgia"/>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="15">
@@ -308,7 +322,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -450,6 +464,11 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -816,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I136"/>
+  <dimension ref="B2:H136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -829,7 +848,6 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="72" t="inlineStr">
         <is>
@@ -844,7 +862,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="63" t="inlineStr">
         <is>
@@ -989,7 +1006,6 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" s="63" t="inlineStr">
         <is>
@@ -1074,7 +1090,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="63" t="inlineStr">
         <is>
@@ -1427,7 +1442,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="B39" s="63" t="inlineStr">
         <is>
@@ -1527,7 +1541,6 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="B47" s="63" t="inlineStr">
         <is>
@@ -1597,7 +1610,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="B53" s="63" t="inlineStr">
         <is>
@@ -1753,7 +1765,6 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="B63" s="63" t="inlineStr">
         <is>
@@ -1860,7 +1871,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="B72" s="64" t="inlineStr">
         <is>
@@ -1868,7 +1878,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
     <row r="74">
       <c r="B74" s="63" t="inlineStr">
         <is>
@@ -8478,7 +8487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H41"/>
+  <dimension ref="B2:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8489,6 +8498,7 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -8504,6 +8514,11 @@
           <t>Layer 3 optional unhedged assertion sites [R]/[G]/[C] (corpus-wide).</t>
         </is>
       </c>
+      <c r="I3" s="74" t="inlineStr">
+        <is>
+          <t>Illustrative only; reverse-test examples, not observed corpus hedges.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
@@ -8541,6 +8556,11 @@
           <t>Coder Notes</t>
         </is>
       </c>
+      <c r="I4" s="75" t="inlineStr">
+        <is>
+          <t>Example hedge (illustrative)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="B5" s="5" t="inlineStr">
@@ -8576,6 +8596,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I5" s="76" t="inlineStr">
+        <is>
+          <t>appeared to reveal / may reveal</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="B6" s="6" t="inlineStr">
@@ -8611,6 +8636,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I6" s="76" t="inlineStr">
+        <is>
+          <t>there appeared to be no zone of inhibition</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="B7" s="5" t="inlineStr">
@@ -8646,6 +8676,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I7" s="76" t="inlineStr">
+        <is>
+          <t>appeared to reveal / may reveal</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="B8" s="6" t="inlineStr">
@@ -8681,6 +8716,11 @@
           <t>Unhedged clause [G] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I8" s="76" t="inlineStr">
+        <is>
+          <t>may not apply / do not necessarily apply</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="B9" s="5" t="inlineStr">
@@ -8716,6 +8756,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I9" s="76" t="inlineStr">
+        <is>
+          <t>appeared to show / suggested</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="B10" s="6" t="inlineStr">
@@ -8751,6 +8796,11 @@
           <t>Unhedged clause [C] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I10" s="76" t="inlineStr">
+        <is>
+          <t>may have caused / appeared to cause</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
@@ -8786,6 +8836,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I11" s="76" t="inlineStr">
+        <is>
+          <t>appeared to reveal / may reveal</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="B12" s="6" t="inlineStr">
@@ -8821,6 +8876,11 @@
           <t>Unhedged clause [G] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I12" s="76" t="inlineStr">
+        <is>
+          <t>may provide / appears to provide</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="B13" s="5" t="inlineStr">
@@ -8856,6 +8916,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I13" s="76" t="inlineStr">
+        <is>
+          <t>appear to exhibit / may exhibit</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="B14" s="6" t="inlineStr">
@@ -8891,6 +8956,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I14" s="76" t="inlineStr">
+        <is>
+          <t>appeared to be / may have been</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="B15" s="5" t="inlineStr">
@@ -8926,6 +8996,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I15" s="76" t="inlineStr">
+        <is>
+          <t>appeared to reveal / may reveal</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="B16" s="6" t="inlineStr">
@@ -8961,6 +9036,11 @@
           <t>Unhedged clause [C] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I16" s="76" t="inlineStr">
+        <is>
+          <t>appeared to achieve / may have achieved</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="B17" s="5" t="inlineStr">
@@ -8996,6 +9076,11 @@
           <t>Unhedged clause [C] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I17" s="76" t="inlineStr">
+        <is>
+          <t>appeared to show / suggested</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="B18" s="6" t="inlineStr">
@@ -9031,6 +9116,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I18" s="76" t="inlineStr">
+        <is>
+          <t>appeared to indicate / may indicate</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="B19" s="5" t="inlineStr">
@@ -9066,6 +9156,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I19" s="76" t="inlineStr">
+        <is>
+          <t>appeared to find / may suggest</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="B20" s="6" t="inlineStr">
@@ -9101,6 +9196,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I20" s="76" t="inlineStr">
+        <is>
+          <t>appeared to be / may have been</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="B21" s="5" t="inlineStr">
@@ -9136,6 +9236,11 @@
           <t>Unhedged clause [G] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I21" s="76" t="inlineStr">
+        <is>
+          <t>appeared to be / may have been</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="B22" s="6" t="inlineStr">
@@ -9171,6 +9276,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I22" s="76" t="inlineStr">
+        <is>
+          <t>appeared to show / suggested</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="B23" s="5" t="inlineStr">
@@ -9206,6 +9316,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I23" s="76" t="inlineStr">
+        <is>
+          <t>appeared to be / may have been</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="B24" s="6" t="inlineStr">
@@ -9241,6 +9356,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I24" s="76" t="inlineStr">
+        <is>
+          <t>appeared to reveal / may reveal</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="45" customHeight="1">
       <c r="B25" s="5" t="inlineStr">
@@ -9276,6 +9396,11 @@
           <t>Unhedged clause [G] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I25" s="76" t="inlineStr">
+        <is>
+          <t>may have / appears to have</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="45" customHeight="1">
       <c r="B26" s="6" t="inlineStr">
@@ -9311,6 +9436,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I26" s="76" t="inlineStr">
+        <is>
+          <t>appeared to exhibit / may have exhibited</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="B27" s="5" t="inlineStr">
@@ -9346,6 +9476,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I27" s="76" t="inlineStr">
+        <is>
+          <t>appeared to find / may suggest</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="45" customHeight="1">
       <c r="B28" s="6" t="inlineStr">
@@ -9381,6 +9516,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I28" s="76" t="inlineStr">
+        <is>
+          <t>appeared to indicate / may indicate</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="45" customHeight="1">
       <c r="B29" s="5" t="inlineStr">
@@ -9416,6 +9556,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I29" s="76" t="inlineStr">
+        <is>
+          <t>appeared to confirm / may confirm</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="B30" s="6" t="inlineStr">
@@ -9451,6 +9596,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I30" s="76" t="inlineStr">
+        <is>
+          <t>there appeared to be no significant difference</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="B31" s="5" t="inlineStr">
@@ -9486,6 +9636,11 @@
           <t>Unhedged clause [G] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I31" s="76" t="inlineStr">
+        <is>
+          <t>may have influenced / appeared to influence</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="45" customHeight="1">
       <c r="B32" s="6" t="inlineStr">
@@ -9521,6 +9676,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I32" s="76" t="inlineStr">
+        <is>
+          <t>appeared to reveal / may reveal</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="45" customHeight="1">
       <c r="B33" s="5" t="inlineStr">
@@ -9556,6 +9716,11 @@
           <t>Unhedged clause [G] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I33" s="76" t="inlineStr">
+        <is>
+          <t>appeared to be / may have been</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="45" customHeight="1">
       <c r="B34" s="6" t="inlineStr">
@@ -9591,6 +9756,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I34" s="76" t="inlineStr">
+        <is>
+          <t>appeared to reveal / may reveal</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="45" customHeight="1">
       <c r="B35" s="5" t="inlineStr">
@@ -9626,6 +9796,11 @@
           <t>Unhedged clause [G] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I35" s="76" t="inlineStr">
+        <is>
+          <t>appeared to be / may have been</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="45" customHeight="1">
       <c r="B36" s="6" t="inlineStr">
@@ -9661,6 +9836,11 @@
           <t>Unhedged clause [C] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I36" s="76" t="inlineStr">
+        <is>
+          <t>appeared to have / may have had</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="45" customHeight="1">
       <c r="B37" s="5" t="inlineStr">
@@ -9696,6 +9876,11 @@
           <t>Unhedged clause [G] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I37" s="76" t="inlineStr">
+        <is>
+          <t>appeared to show / suggested</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="45" customHeight="1">
       <c r="B38" s="6" t="inlineStr">
@@ -9731,6 +9916,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I38" s="76" t="inlineStr">
+        <is>
+          <t>appeared to find / may suggest</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="45" customHeight="1">
       <c r="B39" s="5" t="inlineStr">
@@ -9766,6 +9956,11 @@
           <t>Unhedged clause [G] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I39" s="76" t="inlineStr">
+        <is>
+          <t>suggested / appeared to show</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="45" customHeight="1">
       <c r="B40" s="6" t="inlineStr">
@@ -9801,6 +9996,11 @@
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
         </is>
       </c>
+      <c r="I40" s="76" t="inlineStr">
+        <is>
+          <t>appeared to disclose / suggested</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="45" customHeight="1">
       <c r="B41" s="5" t="inlineStr">
@@ -9834,6 +10034,11 @@
       <c r="H41" s="21" t="inlineStr">
         <is>
           <t>Unhedged clause [R] (sentence-level mark, curated). Reverse test: a hedge could be inserted without changing the facts.</t>
+        </is>
+      </c>
+      <c r="I41" s="76" t="inlineStr">
+        <is>
+          <t>appeared not to be significant</t>
         </is>
       </c>
     </row>

</xml_diff>